<commit_message>
Clean model18altered.xlsx in place; remove separate model18_clean copy
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18altered.xlsx
+++ b/LULU/model18altered.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="56">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -346,6 +346,24 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -405,7 +423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -748,6 +766,24 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="54" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="55" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1115,20 +1151,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B25"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>GLOBAL INVESTMENT SOCIETY  |  INVESTMENT RESEARCH DIVISION</t>
-        </is>
-      </c>
-    </row>
+          <t>GLOBAL INVESTMENT SOCIETY | INVESTMENT RESEARCH DIVISION</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1143,13 +1181,15 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Recommendation:  LONG / OVERWEIGHT</t>
-        </is>
-      </c>
-    </row>
+          <t>Recommendation: LONG / OVERWEIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1160,24 +1200,25 @@
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Blue font  =  figures reported by the company (click value or source link)</t>
+          <t>Blue font = figures reported by the company (click value or source link)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Black font  =  calculations / formulas</t>
+          <t>Black font = calculations / formulas</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions — cols B/C/D on every tab: Justification | Source | Ctrl+F</t>
-        </is>
-      </c>
-    </row>
+          <t>Red font = analyst assumptions — cols B/C/D on every tab: Justification | Source | Ctrl+F</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -1188,7 +1229,7 @@
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>WACC  •  Revenue Drivers  •  NOPAT Bridge  •  Scenarios  •  DCF  •  Comps / Football Field</t>
+          <t>WACC • Revenue Drivers • NOPAT Bridge • Scenarios • DCF • Comps / Football Field</t>
         </is>
       </c>
     </row>
@@ -1207,6 +1248,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1246,6 +1288,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -1300,7 +1343,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
+          <t>Justification (~20 words) [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
@@ -1389,6 +1432,7 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1500,7 +1544,7 @@
     <row r="12">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
+          <t>memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
         </is>
       </c>
     </row>
@@ -1540,6 +1584,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1769,23 +1814,7 @@
       <c r="D25" s="19" t="inlineStr">
         <is>
           <t>YAHOO KEY STATISTICS; βL + debt + equity on ONE page
-(No vendor publishes the D/E embedded inside the regression.)
-Observed levered βL
-  Ctrl+F "Beta (5Y Monthly)"  →  0.86
-  ~60 monthly returns vs S&amp;P 500 (Yahoo label)
-Paired inputs on same page (mrq = most recent quarter)
-  Ctrl+F "Total Debt (mrq)"  →  2.14B
-  Ctrl+F "Market Cap"  →  11.14B
-  Ctrl+F "Total Debt/Equity (mrq)"  →  44.69%  (book; reference only)
-STEP 1 — UNLEVER (market D/E from Yahoo page)
-  D/E = Total Debt (mrq) ÷ Market Cap = 2.14 ÷ 11.14 ≈  0.19
-  βu = 0.86 ÷ [1 + 0.70 × 0.19] = 0.86 ÷ 1.134  ≈  0.76
-  (1−T) = 0.70 at 30% tax on this tab
-STEP 2 — RELEVER (WACC: FY25 10-K lease debt / our market cap)
-  Ctrl+F "Current lease liabilities"  →  298,724
-  Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  D/E ≈ 0.16.  β used = 0.76 × 1.113  ≈  0.84
-Benchmark (not used): Damodaran Retail βu 0.95</t>
+(No vendor publishes the D/E embedded inside the regression.) Observed levered βL Ctrl+F "Beta (5Y Monthly)" → 0.86 ~60 monthly returns vs S&amp;P 500 (Yahoo label) Paired inputs on same page (mrq = most recent quarter) Ctrl+F "Total Debt (mrq)" → 2.14B Ctrl+F "Market Cap" → 11.14B Ctrl+F "Total Debt/Equity (mrq)" → 44.69% (book; reference only) STEP 1 — UNLEVER (market D/E from Yahoo page) D/E = Total Debt (mrq) ÷ Market Cap = 2.14 ÷ 11.14 ≈ 0.19 βu = 0.86 ÷ [1 + 0.70 × 0.19] = 0.86 ÷ 1.134 ≈ 0.76 (1−T) = 0.70 at 30% tax on this tab STEP 2 — RELEVER (WACC: FY25 10-K lease debt / our market cap) Ctrl+F "Current lease liabilities" → 298,724 Ctrl+F "Non-current lease liabilities" → 1,499,717 D/E ≈ 0.16. β used = 0.76 × 1.113 ≈ 0.84 Benchmark (not used): Damodaran Retail βu 0.95</t>
         </is>
       </c>
       <c r="E25" s="29">
@@ -1796,35 +1825,35 @@
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  β walkthrough (Hamada; Yahoo Key Statistics source):</t>
+          <t>β walkthrough (Hamada; Yahoo Key Statistics source):</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (0) Yahoo βL = 0.86 (Beta 5Y Monthly). No vendor publishes D/E inside the regression.</t>
+          <t>(0) Yahoo βL = 0.86 (Beta 5Y Monthly). No vendor publishes D/E inside the regression.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (1) Unlever at Yahoo market D/E = $2.14B debt (mrq) ÷ $11.14B mkt cap ≈ 0.19 → βu ≈ 0.76.</t>
+          <t>(1) Unlever at Yahoo market D/E = $2.14B debt (mrq) ÷ $11.14B mkt cap ≈ 0.19 → βu ≈ 0.76.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2) Relever at WACC D/E = FY25 10-K leases ÷ our market cap ≈ 0.16 → β used ≈ 0.84.</t>
+          <t>(2) Relever at WACC D/E = FY25 10-K leases ÷ our market cap ≈ 0.16 → β used ≈ 0.84.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Book D/E 44.69% on Yahoo page is reference only (not used in formula).</t>
+          <t>Book D/E 44.69% on Yahoo page is reference only (not used in formula).</t>
         </is>
       </c>
     </row>
@@ -1846,6 +1875,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1889,6 +1919,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2038,7 +2069,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
+          <t>Justification (~20 words) [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
@@ -2070,7 +2101,7 @@
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 revenue guide; model −6.1% midpoint</t>
+          <t>Ctrl+F "Q2 FY2026 Management Guidance" → FY2026 revenue guide; model −6.1% midpoint</t>
         </is>
       </c>
       <c r="F4" s="20" t="n">
@@ -2132,7 +2163,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "18.8%" (Q2 OM) and "560 basis points" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".</t>
+          <t>Ctrl+F "Q2 FY2026 Earnings Release (tariff-adjusted margin)" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".</t>
         </is>
       </c>
       <c r="F6" s="20" t="n">
@@ -2163,7 +2194,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
+          <t>Ctrl+F "Q2 FY2026 IEEPA Tariff Refund Disclosure" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
       <c r="F7" s="37" t="n">
@@ -2319,7 +2350,7 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "Net revenue" 11,102,600 = 4.5%.</t>
+          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "FY2025 Form 10-K — Consolidated Revenue = 4.5%.</t>
         </is>
       </c>
       <c r="F12" s="20" t="n">
@@ -2352,18 +2383,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>FY25 actual (10-K)
-  Ctrl+F "680,802"  →  capex $680.8M
-  Ctrl+F "11,102,600"  →  sales $11.1B
-  680.8 / 11,102.6 = 6.1%
-FY26 capex (10-K)
-  Ctrl+F "$725.0 million and $745.0 million"  →  mid $735M
-FY26 sales (earnings)
-  Ctrl+F "$10.350 billion to $10.500 billion"  →  $10.35–$10.50B (mid $10.425B)
-  7.0% = $735M / $10.425B    ($10B year, not FY25 $11.1B)
-DCF blend
-  Fade  7.0 / 6.0 / 5.5 / 5.0 / 4.0
-  5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
+          <t>FY25 actual (10-K) Ctrl+F "680,802" → capex $680.8M Ctrl+F "11,102,600" → sales $11.1B 680.8 / 11,102.6 = 6.1% FY26 capex (10-K) Ctrl+F "$725.0 million and $745.0 million" → mid $735M FY26 sales (earnings) Ctrl+F "$10.350 billion to $10.500 billion" → $10.35–$10.50B (mid $10.425B) 7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B) DCF blend Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0 5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
@@ -2462,8 +2482,7 @@
       <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Not % of revenue; DIO (days).
-FY25 anchor: DIO = (Inventories ÷ COGS) × 365
-  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
+FY25 anchor: DIO = (Inventories ÷ COGS) × 365 = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
 Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.</t>
         </is>
       </c>
@@ -2475,13 +2494,11 @@
       <c r="D16" s="19" t="inlineStr">
         <is>
           <t>Not % of revenue; DIO (days).
-FY25 anchor formula:
-  DIO = (Inventories ÷ COGS) × 365
+FY25 anchor formula: DIO = (Inventories ÷ COGS) × 365
 Ctrl+F "Inventories"
-→ 1,700,753 ($000)  |  FY24: 1,442,081
+→ 1,700,753 ($000) | FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
+→ 4,818,468 ($000) = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
 Forecast: DIO_t = FY25 DIO − (1 × year t)</t>
         </is>
       </c>
@@ -2669,6 +2686,7 @@
         <v>0.75</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -2679,7 +2697,7 @@
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 1</t>
+          <t>Revenue – year 1</t>
         </is>
       </c>
       <c r="F25" s="42">
@@ -2698,7 +2716,7 @@
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 2</t>
+          <t>Revenue – year 2</t>
         </is>
       </c>
       <c r="F26" s="42">
@@ -2717,7 +2735,7 @@
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 3</t>
+          <t>Revenue – year 3</t>
         </is>
       </c>
       <c r="F27" s="42">
@@ -2736,7 +2754,7 @@
     <row r="28">
       <c r="A28" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 4</t>
+          <t>Revenue – year 4</t>
         </is>
       </c>
       <c r="F28" s="42">
@@ -2755,7 +2773,7 @@
     <row r="29">
       <c r="A29" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 5</t>
+          <t>Revenue – year 5</t>
         </is>
       </c>
       <c r="F29" s="42">
@@ -2774,7 +2792,7 @@
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gross margin % – year 1</t>
+          <t>Gross margin % – year 1</t>
         </is>
       </c>
       <c r="F30" s="43">
@@ -2793,7 +2811,7 @@
     <row r="31">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gross margin % – year 2</t>
+          <t>Gross margin % – year 2</t>
         </is>
       </c>
       <c r="F31" s="43">
@@ -2812,7 +2830,7 @@
     <row r="32">
       <c r="A32" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gross margin % – year 3</t>
+          <t>Gross margin % – year 3</t>
         </is>
       </c>
       <c r="F32" s="43">
@@ -2831,7 +2849,7 @@
     <row r="33">
       <c r="A33" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gross margin % – year 4</t>
+          <t>Gross margin % – year 4</t>
         </is>
       </c>
       <c r="F33" s="43">
@@ -2850,7 +2868,7 @@
     <row r="34">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gross margin % – year 5</t>
+          <t>Gross margin % – year 5</t>
         </is>
       </c>
       <c r="F34" s="43">
@@ -2869,7 +2887,7 @@
     <row r="35">
       <c r="A35" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost of goods sold (COGS) – year 1</t>
+          <t>Cost of goods sold (COGS) – year 1</t>
         </is>
       </c>
       <c r="F35" s="42">
@@ -2888,7 +2906,7 @@
     <row r="36">
       <c r="A36" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost of goods sold (COGS) – year 2</t>
+          <t>Cost of goods sold (COGS) – year 2</t>
         </is>
       </c>
       <c r="F36" s="42">
@@ -2907,7 +2925,7 @@
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost of goods sold (COGS) – year 3</t>
+          <t>Cost of goods sold (COGS) – year 3</t>
         </is>
       </c>
       <c r="F37" s="42">
@@ -2926,7 +2944,7 @@
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost of goods sold (COGS) – year 4</t>
+          <t>Cost of goods sold (COGS) – year 4</t>
         </is>
       </c>
       <c r="F38" s="42">
@@ -2945,7 +2963,7 @@
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost of goods sold (COGS) – year 5</t>
+          <t>Cost of goods sold (COGS) – year 5</t>
         </is>
       </c>
       <c r="F39" s="42">
@@ -2964,7 +2982,7 @@
     <row r="40">
       <c r="A40" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 1</t>
+          <t>Clean EBIT margin – year 1</t>
         </is>
       </c>
       <c r="F40" s="43">
@@ -2983,7 +3001,7 @@
     <row r="41">
       <c r="A41" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 2</t>
+          <t>Clean EBIT margin – year 2</t>
         </is>
       </c>
       <c r="F41" s="43">
@@ -3002,7 +3020,7 @@
     <row r="42">
       <c r="A42" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 3</t>
+          <t>Clean EBIT margin – year 3</t>
         </is>
       </c>
       <c r="F42" s="43">
@@ -3021,7 +3039,7 @@
     <row r="43">
       <c r="A43" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 4</t>
+          <t>Clean EBIT margin – year 4</t>
         </is>
       </c>
       <c r="F43" s="43">
@@ -3040,7 +3058,7 @@
     <row r="44">
       <c r="A44" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 5</t>
+          <t>Clean EBIT margin – year 5</t>
         </is>
       </c>
       <c r="F44" s="43">
@@ -3059,7 +3077,7 @@
     <row r="45">
       <c r="A45" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 1</t>
+          <t>EBIT – year 1</t>
         </is>
       </c>
       <c r="F45" s="42">
@@ -3078,7 +3096,7 @@
     <row r="46">
       <c r="A46" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 2</t>
+          <t>EBIT – year 2</t>
         </is>
       </c>
       <c r="F46" s="42">
@@ -3097,7 +3115,7 @@
     <row r="47">
       <c r="A47" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 3</t>
+          <t>EBIT – year 3</t>
         </is>
       </c>
       <c r="F47" s="42">
@@ -3116,7 +3134,7 @@
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 4</t>
+          <t>EBIT – year 4</t>
         </is>
       </c>
       <c r="F48" s="42">
@@ -3135,7 +3153,7 @@
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 5</t>
+          <t>EBIT – year 5</t>
         </is>
       </c>
       <c r="F49" s="42">
@@ -3154,7 +3172,7 @@
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 1</t>
+          <t>NOPAT – year 1</t>
         </is>
       </c>
       <c r="F50" s="42">
@@ -3173,7 +3191,7 @@
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 2</t>
+          <t>NOPAT – year 2</t>
         </is>
       </c>
       <c r="F51" s="42">
@@ -3192,7 +3210,7 @@
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 3</t>
+          <t>NOPAT – year 3</t>
         </is>
       </c>
       <c r="F52" s="42">
@@ -3211,7 +3229,7 @@
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 4</t>
+          <t>NOPAT – year 4</t>
         </is>
       </c>
       <c r="F53" s="42">
@@ -3230,7 +3248,7 @@
     <row r="54">
       <c r="A54" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 5</t>
+          <t>NOPAT – year 5</t>
         </is>
       </c>
       <c r="F54" s="42">
@@ -3249,7 +3267,7 @@
     <row r="55">
       <c r="A55" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 1</t>
+          <t>D&amp;A – year 1</t>
         </is>
       </c>
       <c r="F55" s="42">
@@ -3268,7 +3286,7 @@
     <row r="56">
       <c r="A56" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 2</t>
+          <t>D&amp;A – year 2</t>
         </is>
       </c>
       <c r="F56" s="42">
@@ -3287,7 +3305,7 @@
     <row r="57">
       <c r="A57" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 3</t>
+          <t>D&amp;A – year 3</t>
         </is>
       </c>
       <c r="F57" s="42">
@@ -3306,7 +3324,7 @@
     <row r="58">
       <c r="A58" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 4</t>
+          <t>D&amp;A – year 4</t>
         </is>
       </c>
       <c r="F58" s="42">
@@ -3325,7 +3343,7 @@
     <row r="59">
       <c r="A59" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 5</t>
+          <t>D&amp;A – year 5</t>
         </is>
       </c>
       <c r="F59" s="42">
@@ -3344,7 +3362,7 @@
     <row r="60">
       <c r="A60" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 1</t>
+          <t>Capex – year 1</t>
         </is>
       </c>
       <c r="F60" s="42">
@@ -3363,7 +3381,7 @@
     <row r="61">
       <c r="A61" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 2</t>
+          <t>Capex – year 2</t>
         </is>
       </c>
       <c r="F61" s="42">
@@ -3382,7 +3400,7 @@
     <row r="62">
       <c r="A62" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 3</t>
+          <t>Capex – year 3</t>
         </is>
       </c>
       <c r="F62" s="42">
@@ -3401,7 +3419,7 @@
     <row r="63">
       <c r="A63" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 4</t>
+          <t>Capex – year 4</t>
         </is>
       </c>
       <c r="F63" s="42">
@@ -3420,7 +3438,7 @@
     <row r="64">
       <c r="A64" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 5</t>
+          <t>Capex – year 5</t>
         </is>
       </c>
       <c r="F64" s="42">
@@ -3439,7 +3457,7 @@
     <row r="65">
       <c r="A65" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) – year 1</t>
+          <t>DSO (days) – year 1</t>
         </is>
       </c>
       <c r="F65" s="44">
@@ -3458,7 +3476,7 @@
     <row r="66">
       <c r="A66" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) – year 2</t>
+          <t>DSO (days) – year 2</t>
         </is>
       </c>
       <c r="F66" s="44">
@@ -3477,7 +3495,7 @@
     <row r="67">
       <c r="A67" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) – year 3</t>
+          <t>DSO (days) – year 3</t>
         </is>
       </c>
       <c r="F67" s="44">
@@ -3496,7 +3514,7 @@
     <row r="68">
       <c r="A68" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) – year 4</t>
+          <t>DSO (days) – year 4</t>
         </is>
       </c>
       <c r="F68" s="44">
@@ -3515,7 +3533,7 @@
     <row r="69">
       <c r="A69" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) – year 5</t>
+          <t>DSO (days) – year 5</t>
         </is>
       </c>
       <c r="F69" s="44">
@@ -3534,7 +3552,7 @@
     <row r="70">
       <c r="A70" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 1</t>
+          <t>Accounts receivable – year 1</t>
         </is>
       </c>
       <c r="F70" s="42">
@@ -3553,7 +3571,7 @@
     <row r="71">
       <c r="A71" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 2</t>
+          <t>Accounts receivable – year 2</t>
         </is>
       </c>
       <c r="F71" s="42">
@@ -3572,7 +3590,7 @@
     <row r="72">
       <c r="A72" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 3</t>
+          <t>Accounts receivable – year 3</t>
         </is>
       </c>
       <c r="F72" s="42">
@@ -3591,7 +3609,7 @@
     <row r="73">
       <c r="A73" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 4</t>
+          <t>Accounts receivable – year 4</t>
         </is>
       </c>
       <c r="F73" s="42">
@@ -3610,7 +3628,7 @@
     <row r="74">
       <c r="A74" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 5</t>
+          <t>Accounts receivable – year 5</t>
         </is>
       </c>
       <c r="F74" s="42">
@@ -3629,7 +3647,7 @@
     <row r="75">
       <c r="A75" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) – year 1</t>
+          <t>DIO (days) – year 1</t>
         </is>
       </c>
       <c r="F75" s="44">
@@ -3648,7 +3666,7 @@
     <row r="76">
       <c r="A76" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) – year 2</t>
+          <t>DIO (days) – year 2</t>
         </is>
       </c>
       <c r="F76" s="44">
@@ -3667,7 +3685,7 @@
     <row r="77">
       <c r="A77" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) – year 3</t>
+          <t>DIO (days) – year 3</t>
         </is>
       </c>
       <c r="F77" s="44">
@@ -3686,7 +3704,7 @@
     <row r="78">
       <c r="A78" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) – year 4</t>
+          <t>DIO (days) – year 4</t>
         </is>
       </c>
       <c r="F78" s="44">
@@ -3705,7 +3723,7 @@
     <row r="79">
       <c r="A79" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) – year 5</t>
+          <t>DIO (days) – year 5</t>
         </is>
       </c>
       <c r="F79" s="44">
@@ -3724,7 +3742,7 @@
     <row r="80">
       <c r="A80" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories – year 1</t>
+          <t>Inventories – year 1</t>
         </is>
       </c>
       <c r="F80" s="42">
@@ -3743,7 +3761,7 @@
     <row r="81">
       <c r="A81" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories – year 2</t>
+          <t>Inventories – year 2</t>
         </is>
       </c>
       <c r="F81" s="42">
@@ -3762,7 +3780,7 @@
     <row r="82">
       <c r="A82" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories – year 3</t>
+          <t>Inventories – year 3</t>
         </is>
       </c>
       <c r="F82" s="42">
@@ -3781,7 +3799,7 @@
     <row r="83">
       <c r="A83" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories – year 4</t>
+          <t>Inventories – year 4</t>
         </is>
       </c>
       <c r="F83" s="42">
@@ -3800,7 +3818,7 @@
     <row r="84">
       <c r="A84" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories – year 5</t>
+          <t>Inventories – year 5</t>
         </is>
       </c>
       <c r="F84" s="42">
@@ -3819,7 +3837,7 @@
     <row r="85">
       <c r="A85" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) – year 1</t>
+          <t>DPO (days) – year 1</t>
         </is>
       </c>
       <c r="F85" s="44">
@@ -3838,7 +3856,7 @@
     <row r="86">
       <c r="A86" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) – year 2</t>
+          <t>DPO (days) – year 2</t>
         </is>
       </c>
       <c r="F86" s="44">
@@ -3857,7 +3875,7 @@
     <row r="87">
       <c r="A87" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) – year 3</t>
+          <t>DPO (days) – year 3</t>
         </is>
       </c>
       <c r="F87" s="44">
@@ -3876,7 +3894,7 @@
     <row r="88">
       <c r="A88" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) – year 4</t>
+          <t>DPO (days) – year 4</t>
         </is>
       </c>
       <c r="F88" s="44">
@@ -3895,7 +3913,7 @@
     <row r="89">
       <c r="A89" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) – year 5</t>
+          <t>DPO (days) – year 5</t>
         </is>
       </c>
       <c r="F89" s="44">
@@ -3914,7 +3932,7 @@
     <row r="90">
       <c r="A90" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable – year 1</t>
+          <t>Accounts payable – year 1</t>
         </is>
       </c>
       <c r="F90" s="42">
@@ -3933,7 +3951,7 @@
     <row r="91">
       <c r="A91" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable – year 2</t>
+          <t>Accounts payable – year 2</t>
         </is>
       </c>
       <c r="F91" s="42">
@@ -3952,7 +3970,7 @@
     <row r="92">
       <c r="A92" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable – year 3</t>
+          <t>Accounts payable – year 3</t>
         </is>
       </c>
       <c r="F92" s="42">
@@ -3971,7 +3989,7 @@
     <row r="93">
       <c r="A93" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable – year 4</t>
+          <t>Accounts payable – year 4</t>
         </is>
       </c>
       <c r="F93" s="42">
@@ -3990,7 +4008,7 @@
     <row r="94">
       <c r="A94" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable – year 5</t>
+          <t>Accounts payable – year 5</t>
         </is>
       </c>
       <c r="F94" s="42">
@@ -4009,7 +4027,7 @@
     <row r="95">
       <c r="A95" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets) – year 1</t>
+          <t>Prepaid expenses (other current assets) – year 1</t>
         </is>
       </c>
       <c r="F95" s="42">
@@ -4028,7 +4046,7 @@
     <row r="96">
       <c r="A96" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets) – year 2</t>
+          <t>Prepaid expenses (other current assets) – year 2</t>
         </is>
       </c>
       <c r="F96" s="42">
@@ -4047,7 +4065,7 @@
     <row r="97">
       <c r="A97" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets) – year 3</t>
+          <t>Prepaid expenses (other current assets) – year 3</t>
         </is>
       </c>
       <c r="F97" s="42">
@@ -4066,7 +4084,7 @@
     <row r="98">
       <c r="A98" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets) – year 4</t>
+          <t>Prepaid expenses (other current assets) – year 4</t>
         </is>
       </c>
       <c r="F98" s="42">
@@ -4085,7 +4103,7 @@
     <row r="99">
       <c r="A99" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets) – year 5</t>
+          <t>Prepaid expenses (other current assets) – year 5</t>
         </is>
       </c>
       <c r="F99" s="42">
@@ -4104,7 +4122,7 @@
     <row r="100">
       <c r="A100" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities – year 1</t>
+          <t>Accrued liabilities – year 1</t>
         </is>
       </c>
       <c r="F100" s="42">
@@ -4123,7 +4141,7 @@
     <row r="101">
       <c r="A101" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities – year 2</t>
+          <t>Accrued liabilities – year 2</t>
         </is>
       </c>
       <c r="F101" s="42">
@@ -4142,7 +4160,7 @@
     <row r="102">
       <c r="A102" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities – year 3</t>
+          <t>Accrued liabilities – year 3</t>
         </is>
       </c>
       <c r="F102" s="42">
@@ -4161,7 +4179,7 @@
     <row r="103">
       <c r="A103" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities – year 4</t>
+          <t>Accrued liabilities – year 4</t>
         </is>
       </c>
       <c r="F103" s="42">
@@ -4180,7 +4198,7 @@
     <row r="104">
       <c r="A104" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities – year 5</t>
+          <t>Accrued liabilities – year 5</t>
         </is>
       </c>
       <c r="F104" s="42">
@@ -4199,7 +4217,7 @@
     <row r="105">
       <c r="A105" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating assets (AR + inv + prepaids) – year 1</t>
+          <t>Current operating assets (AR + inv + prepaids) – year 1</t>
         </is>
       </c>
       <c r="F105" s="42">
@@ -4218,7 +4236,7 @@
     <row r="106">
       <c r="A106" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating assets (AR + inv + prepaids) – year 2</t>
+          <t>Current operating assets (AR + inv + prepaids) – year 2</t>
         </is>
       </c>
       <c r="F106" s="42">
@@ -4237,7 +4255,7 @@
     <row r="107">
       <c r="A107" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating assets (AR + inv + prepaids) – year 3</t>
+          <t>Current operating assets (AR + inv + prepaids) – year 3</t>
         </is>
       </c>
       <c r="F107" s="42">
@@ -4256,7 +4274,7 @@
     <row r="108">
       <c r="A108" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating assets (AR + inv + prepaids) – year 4</t>
+          <t>Current operating assets (AR + inv + prepaids) – year 4</t>
         </is>
       </c>
       <c r="F108" s="42">
@@ -4275,7 +4293,7 @@
     <row r="109">
       <c r="A109" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating assets (AR + inv + prepaids) – year 5</t>
+          <t>Current operating assets (AR + inv + prepaids) – year 5</t>
         </is>
       </c>
       <c r="F109" s="42">
@@ -4294,7 +4312,7 @@
     <row r="110">
       <c r="A110" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating liabilities (AP + accruals) – year 1</t>
+          <t>Current operating liabilities (AP + accruals) – year 1</t>
         </is>
       </c>
       <c r="F110" s="42">
@@ -4313,7 +4331,7 @@
     <row r="111">
       <c r="A111" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating liabilities (AP + accruals) – year 2</t>
+          <t>Current operating liabilities (AP + accruals) – year 2</t>
         </is>
       </c>
       <c r="F111" s="42">
@@ -4332,7 +4350,7 @@
     <row r="112">
       <c r="A112" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating liabilities (AP + accruals) – year 3</t>
+          <t>Current operating liabilities (AP + accruals) – year 3</t>
         </is>
       </c>
       <c r="F112" s="42">
@@ -4351,7 +4369,7 @@
     <row r="113">
       <c r="A113" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating liabilities (AP + accruals) – year 4</t>
+          <t>Current operating liabilities (AP + accruals) – year 4</t>
         </is>
       </c>
       <c r="F113" s="42">
@@ -4370,7 +4388,7 @@
     <row r="114">
       <c r="A114" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Current operating liabilities (AP + accruals) – year 5</t>
+          <t>Current operating liabilities (AP + accruals) – year 5</t>
         </is>
       </c>
       <c r="F114" s="42">
@@ -4389,7 +4407,7 @@
     <row r="115">
       <c r="A115" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net working capital – year 1</t>
+          <t>Net working capital – year 1</t>
         </is>
       </c>
       <c r="F115" s="42">
@@ -4408,7 +4426,7 @@
     <row r="116">
       <c r="A116" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net working capital – year 2</t>
+          <t>Net working capital – year 2</t>
         </is>
       </c>
       <c r="F116" s="42">
@@ -4427,7 +4445,7 @@
     <row r="117">
       <c r="A117" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net working capital – year 3</t>
+          <t>Net working capital – year 3</t>
         </is>
       </c>
       <c r="F117" s="42">
@@ -4446,7 +4464,7 @@
     <row r="118">
       <c r="A118" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net working capital – year 4</t>
+          <t>Net working capital – year 4</t>
         </is>
       </c>
       <c r="F118" s="42">
@@ -4465,7 +4483,7 @@
     <row r="119">
       <c r="A119" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net working capital – year 5</t>
+          <t>Net working capital – year 5</t>
         </is>
       </c>
       <c r="F119" s="42">
@@ -4484,7 +4502,7 @@
     <row r="120">
       <c r="A120" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC (prior yr − current yr) – year 1</t>
+          <t>ΔNWC (prior yr − current yr) – year 1</t>
         </is>
       </c>
       <c r="F120" s="42">
@@ -4503,7 +4521,7 @@
     <row r="121">
       <c r="A121" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC (prior yr − current yr) – year 2</t>
+          <t>ΔNWC (prior yr − current yr) – year 2</t>
         </is>
       </c>
       <c r="F121" s="42">
@@ -4522,7 +4540,7 @@
     <row r="122">
       <c r="A122" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC (prior yr − current yr) – year 3</t>
+          <t>ΔNWC (prior yr − current yr) – year 3</t>
         </is>
       </c>
       <c r="F122" s="42">
@@ -4541,7 +4559,7 @@
     <row r="123">
       <c r="A123" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC (prior yr − current yr) – year 4</t>
+          <t>ΔNWC (prior yr − current yr) – year 4</t>
         </is>
       </c>
       <c r="F123" s="42">
@@ -4560,7 +4578,7 @@
     <row r="124">
       <c r="A124" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC (prior yr − current yr) – year 5</t>
+          <t>ΔNWC (prior yr − current yr) – year 5</t>
         </is>
       </c>
       <c r="F124" s="42">
@@ -4579,7 +4597,7 @@
     <row r="125">
       <c r="A125" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 1</t>
+          <t>Unlevered FCF – year 1</t>
         </is>
       </c>
       <c r="F125" s="42">
@@ -4598,7 +4616,7 @@
     <row r="126">
       <c r="A126" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 2</t>
+          <t>Unlevered FCF – year 2</t>
         </is>
       </c>
       <c r="F126" s="42">
@@ -4617,7 +4635,7 @@
     <row r="127">
       <c r="A127" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 3</t>
+          <t>Unlevered FCF – year 3</t>
         </is>
       </c>
       <c r="F127" s="42">
@@ -4636,7 +4654,7 @@
     <row r="128">
       <c r="A128" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 4</t>
+          <t>Unlevered FCF – year 4</t>
         </is>
       </c>
       <c r="F128" s="42">
@@ -4655,7 +4673,7 @@
     <row r="129">
       <c r="A129" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 5</t>
+          <t>Unlevered FCF – year 5</t>
         </is>
       </c>
       <c r="F129" s="42">
@@ -4671,6 +4689,7 @@
         <v/>
       </c>
     </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4728,6 +4747,7 @@
         <v/>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4735,6 +4755,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -4745,7 +4766,7 @@
     <row r="138">
       <c r="A138" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other income – year 1</t>
+          <t>Other income – year 1</t>
         </is>
       </c>
       <c r="F138" s="42" t="n">
@@ -4761,7 +4782,7 @@
     <row r="139">
       <c r="A139" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other income – year 2</t>
+          <t>Other income – year 2</t>
         </is>
       </c>
       <c r="F139" s="42" t="n">
@@ -4777,7 +4798,7 @@
     <row r="140">
       <c r="A140" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other income – year 3</t>
+          <t>Other income – year 3</t>
         </is>
       </c>
       <c r="F140" s="42" t="n">
@@ -4793,7 +4814,7 @@
     <row r="141">
       <c r="A141" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other income – year 4</t>
+          <t>Other income – year 4</t>
         </is>
       </c>
       <c r="F141" s="42" t="n">
@@ -4809,7 +4830,7 @@
     <row r="142">
       <c r="A142" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other income – year 5</t>
+          <t>Other income – year 5</t>
         </is>
       </c>
       <c r="F142" s="42" t="n">
@@ -4825,7 +4846,7 @@
     <row r="143">
       <c r="A143" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net income – year 1</t>
+          <t>Net income – year 1</t>
         </is>
       </c>
       <c r="F143" s="42">
@@ -4844,7 +4865,7 @@
     <row r="144">
       <c r="A144" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net income – year 2</t>
+          <t>Net income – year 2</t>
         </is>
       </c>
       <c r="F144" s="42">
@@ -4863,7 +4884,7 @@
     <row r="145">
       <c r="A145" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net income – year 3</t>
+          <t>Net income – year 3</t>
         </is>
       </c>
       <c r="F145" s="42">
@@ -4882,7 +4903,7 @@
     <row r="146">
       <c r="A146" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net income – year 4</t>
+          <t>Net income – year 4</t>
         </is>
       </c>
       <c r="F146" s="42">
@@ -4901,7 +4922,7 @@
     <row r="147">
       <c r="A147" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net income – year 5</t>
+          <t>Net income – year 5</t>
         </is>
       </c>
       <c r="F147" s="42">
@@ -4920,7 +4941,7 @@
     <row r="148">
       <c r="A148" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash from operations – year 1</t>
+          <t>Cash from operations – year 1</t>
         </is>
       </c>
       <c r="F148" s="42">
@@ -4939,7 +4960,7 @@
     <row r="149">
       <c r="A149" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash from operations – year 2</t>
+          <t>Cash from operations – year 2</t>
         </is>
       </c>
       <c r="F149" s="42">
@@ -4958,7 +4979,7 @@
     <row r="150">
       <c r="A150" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash from operations – year 3</t>
+          <t>Cash from operations – year 3</t>
         </is>
       </c>
       <c r="F150" s="42">
@@ -4977,7 +4998,7 @@
     <row r="151">
       <c r="A151" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash from operations – year 4</t>
+          <t>Cash from operations – year 4</t>
         </is>
       </c>
       <c r="F151" s="42">
@@ -4996,7 +5017,7 @@
     <row r="152">
       <c r="A152" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash from operations – year 5</t>
+          <t>Cash from operations – year 5</t>
         </is>
       </c>
       <c r="F152" s="42">
@@ -5015,7 +5036,7 @@
     <row r="153">
       <c r="A153" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Free cash flow (CFS) – year 1</t>
+          <t>Free cash flow (CFS) – year 1</t>
         </is>
       </c>
       <c r="F153" s="42">
@@ -5034,7 +5055,7 @@
     <row r="154">
       <c r="A154" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Free cash flow (CFS) – year 2</t>
+          <t>Free cash flow (CFS) – year 2</t>
         </is>
       </c>
       <c r="F154" s="42">
@@ -5053,7 +5074,7 @@
     <row r="155">
       <c r="A155" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Free cash flow (CFS) – year 3</t>
+          <t>Free cash flow (CFS) – year 3</t>
         </is>
       </c>
       <c r="F155" s="42">
@@ -5072,7 +5093,7 @@
     <row r="156">
       <c r="A156" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Free cash flow (CFS) – year 4</t>
+          <t>Free cash flow (CFS) – year 4</t>
         </is>
       </c>
       <c r="F156" s="42">
@@ -5091,7 +5112,7 @@
     <row r="157">
       <c r="A157" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Free cash flow (CFS) – year 5</t>
+          <t>Free cash flow (CFS) – year 5</t>
         </is>
       </c>
       <c r="F157" s="42">
@@ -5110,7 +5131,7 @@
     <row r="158">
       <c r="A158" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Share repurchases – year 1</t>
+          <t>Share repurchases – year 1</t>
         </is>
       </c>
       <c r="F158" s="42">
@@ -5129,7 +5150,7 @@
     <row r="159">
       <c r="A159" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Share repurchases – year 2</t>
+          <t>Share repurchases – year 2</t>
         </is>
       </c>
       <c r="F159" s="42">
@@ -5148,7 +5169,7 @@
     <row r="160">
       <c r="A160" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Share repurchases – year 3</t>
+          <t>Share repurchases – year 3</t>
         </is>
       </c>
       <c r="F160" s="42">
@@ -5167,7 +5188,7 @@
     <row r="161">
       <c r="A161" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Share repurchases – year 4</t>
+          <t>Share repurchases – year 4</t>
         </is>
       </c>
       <c r="F161" s="42">
@@ -5186,7 +5207,7 @@
     <row r="162">
       <c r="A162" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Share repurchases – year 5</t>
+          <t>Share repurchases – year 5</t>
         </is>
       </c>
       <c r="F162" s="42">
@@ -5205,7 +5226,7 @@
     <row r="163">
       <c r="A163" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash &amp; equivalents – year 1</t>
+          <t>Cash &amp; equivalents – year 1</t>
         </is>
       </c>
       <c r="F163" s="42">
@@ -5224,7 +5245,7 @@
     <row r="164">
       <c r="A164" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash &amp; equivalents – year 2</t>
+          <t>Cash &amp; equivalents – year 2</t>
         </is>
       </c>
       <c r="F164" s="42">
@@ -5243,7 +5264,7 @@
     <row r="165">
       <c r="A165" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash &amp; equivalents – year 3</t>
+          <t>Cash &amp; equivalents – year 3</t>
         </is>
       </c>
       <c r="F165" s="42">
@@ -5262,7 +5283,7 @@
     <row r="166">
       <c r="A166" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash &amp; equivalents – year 4</t>
+          <t>Cash &amp; equivalents – year 4</t>
         </is>
       </c>
       <c r="F166" s="42">
@@ -5281,7 +5302,7 @@
     <row r="167">
       <c r="A167" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash &amp; equivalents – year 5</t>
+          <t>Cash &amp; equivalents – year 5</t>
         </is>
       </c>
       <c r="F167" s="42">
@@ -5300,7 +5321,7 @@
     <row r="168">
       <c r="A168" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total assets – year 1</t>
+          <t>Total assets – year 1</t>
         </is>
       </c>
       <c r="F168" s="42">
@@ -5319,7 +5340,7 @@
     <row r="169">
       <c r="A169" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total assets – year 2</t>
+          <t>Total assets – year 2</t>
         </is>
       </c>
       <c r="F169" s="42">
@@ -5338,7 +5359,7 @@
     <row r="170">
       <c r="A170" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total assets – year 3</t>
+          <t>Total assets – year 3</t>
         </is>
       </c>
       <c r="F170" s="42">
@@ -5357,7 +5378,7 @@
     <row r="171">
       <c r="A171" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total assets – year 4</t>
+          <t>Total assets – year 4</t>
         </is>
       </c>
       <c r="F171" s="42">
@@ -5376,7 +5397,7 @@
     <row r="172">
       <c r="A172" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total assets – year 5</t>
+          <t>Total assets – year 5</t>
         </is>
       </c>
       <c r="F172" s="42">
@@ -5395,7 +5416,7 @@
     <row r="173">
       <c r="A173" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total liabilities – year 1</t>
+          <t>Total liabilities – year 1</t>
         </is>
       </c>
       <c r="F173" s="42">
@@ -5414,7 +5435,7 @@
     <row r="174">
       <c r="A174" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total liabilities – year 2</t>
+          <t>Total liabilities – year 2</t>
         </is>
       </c>
       <c r="F174" s="42">
@@ -5433,7 +5454,7 @@
     <row r="175">
       <c r="A175" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total liabilities – year 3</t>
+          <t>Total liabilities – year 3</t>
         </is>
       </c>
       <c r="F175" s="42">
@@ -5452,7 +5473,7 @@
     <row r="176">
       <c r="A176" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total liabilities – year 4</t>
+          <t>Total liabilities – year 4</t>
         </is>
       </c>
       <c r="F176" s="42">
@@ -5471,7 +5492,7 @@
     <row r="177">
       <c r="A177" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total liabilities – year 5</t>
+          <t>Total liabilities – year 5</t>
         </is>
       </c>
       <c r="F177" s="42">
@@ -5490,7 +5511,7 @@
     <row r="178">
       <c r="A178" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total equity – year 1</t>
+          <t>Total equity – year 1</t>
         </is>
       </c>
       <c r="F178" s="42">
@@ -5509,7 +5530,7 @@
     <row r="179">
       <c r="A179" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total equity – year 2</t>
+          <t>Total equity – year 2</t>
         </is>
       </c>
       <c r="F179" s="42">
@@ -5528,7 +5549,7 @@
     <row r="180">
       <c r="A180" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total equity – year 3</t>
+          <t>Total equity – year 3</t>
         </is>
       </c>
       <c r="F180" s="42">
@@ -5547,7 +5568,7 @@
     <row r="181">
       <c r="A181" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total equity – year 4</t>
+          <t>Total equity – year 4</t>
         </is>
       </c>
       <c r="F181" s="42">
@@ -5566,7 +5587,7 @@
     <row r="182">
       <c r="A182" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total equity – year 5</t>
+          <t>Total equity – year 5</t>
         </is>
       </c>
       <c r="F182" s="42">
@@ -5585,7 +5606,7 @@
     <row r="183">
       <c r="A183" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted shares (000) – year 1</t>
+          <t>Diluted shares (000) – year 1</t>
         </is>
       </c>
       <c r="F183" s="42">
@@ -5604,7 +5625,7 @@
     <row r="184">
       <c r="A184" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted shares (000) – year 2</t>
+          <t>Diluted shares (000) – year 2</t>
         </is>
       </c>
       <c r="F184" s="42">
@@ -5623,7 +5644,7 @@
     <row r="185">
       <c r="A185" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted shares (000) – year 3</t>
+          <t>Diluted shares (000) – year 3</t>
         </is>
       </c>
       <c r="F185" s="42">
@@ -5642,7 +5663,7 @@
     <row r="186">
       <c r="A186" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted shares (000) – year 4</t>
+          <t>Diluted shares (000) – year 4</t>
         </is>
       </c>
       <c r="F186" s="42">
@@ -5661,7 +5682,7 @@
     <row r="187">
       <c r="A187" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted shares (000) – year 5</t>
+          <t>Diluted shares (000) – year 5</t>
         </is>
       </c>
       <c r="F187" s="42">
@@ -5680,7 +5701,7 @@
     <row r="188">
       <c r="A188" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 1</t>
+          <t>Diluted EPS ($) – year 1</t>
         </is>
       </c>
       <c r="F188" s="49">
@@ -5699,7 +5720,7 @@
     <row r="189">
       <c r="A189" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 2</t>
+          <t>Diluted EPS ($) – year 2</t>
         </is>
       </c>
       <c r="F189" s="49">
@@ -5718,7 +5739,7 @@
     <row r="190">
       <c r="A190" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 3</t>
+          <t>Diluted EPS ($) – year 3</t>
         </is>
       </c>
       <c r="F190" s="49">
@@ -5737,7 +5758,7 @@
     <row r="191">
       <c r="A191" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 4</t>
+          <t>Diluted EPS ($) – year 4</t>
         </is>
       </c>
       <c r="F191" s="49">
@@ -5756,7 +5777,7 @@
     <row r="192">
       <c r="A192" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 5</t>
+          <t>Diluted EPS ($) – year 5</t>
         </is>
       </c>
       <c r="F192" s="49">
@@ -5775,7 +5796,7 @@
     <row r="193">
       <c r="A193" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: pitch deck pulls cols G (base) &amp; H (bull) from this block via pitch_values.py</t>
+          <t>memo: pitch deck pulls cols G (base) &amp; H (bull) from this block via pitch_values.py</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5949,7 @@
       </c>
       <c r="J5" s="56" t="inlineStr">
         <is>
-          <t>Justification  [cols I–L: click + to expand]</t>
+          <t>Justification [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K5" s="56" t="inlineStr">
@@ -5945,7 +5966,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas — beginning stores</t>
+          <t>Americas — beginning stores</t>
         </is>
       </c>
       <c r="B6" s="57" t="n">
@@ -5995,7 +6016,7 @@
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas — openings</t>
+          <t>Americas — openings</t>
         </is>
       </c>
       <c r="C7" s="60" t="n">
@@ -6037,7 +6058,7 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas — closures</t>
+          <t>Americas — closures</t>
         </is>
       </c>
       <c r="C8" s="60" t="n">
@@ -6079,7 +6100,7 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas — ending stores</t>
+          <t>Americas — ending stores</t>
         </is>
       </c>
       <c r="B9" s="57" t="n">
@@ -6129,7 +6150,7 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland — beginning stores</t>
+          <t>China Mainland — beginning stores</t>
         </is>
       </c>
       <c r="B10" s="57" t="n">
@@ -6179,7 +6200,7 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland — openings</t>
+          <t>China Mainland — openings</t>
         </is>
       </c>
       <c r="C11" s="60" t="n">
@@ -6221,7 +6242,7 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland — closures</t>
+          <t>China Mainland — closures</t>
         </is>
       </c>
       <c r="C12" s="60" t="n">
@@ -6263,7 +6284,7 @@
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland — ending stores</t>
+          <t>China Mainland — ending stores</t>
         </is>
       </c>
       <c r="B13" s="57" t="n">
@@ -6313,7 +6334,7 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World — beginning stores</t>
+          <t>Rest of World — beginning stores</t>
         </is>
       </c>
       <c r="B14" s="57" t="n">
@@ -6363,7 +6384,7 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World — openings</t>
+          <t>Rest of World — openings</t>
         </is>
       </c>
       <c r="C15" s="60" t="n">
@@ -6405,7 +6426,7 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World — closures</t>
+          <t>Rest of World — closures</t>
         </is>
       </c>
       <c r="C16" s="60" t="n">
@@ -6447,7 +6468,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World — ending stores</t>
+          <t>Rest of World — ending stores</t>
         </is>
       </c>
       <c r="B17" s="57" t="n">
@@ -6635,6 +6656,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6690,7 +6712,7 @@
       </c>
       <c r="J23" s="56" t="inlineStr">
         <is>
-          <t>Justification  [cols I–L: click + to expand]</t>
+          <t>Justification [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K23" s="56" t="inlineStr">
@@ -6752,7 +6774,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas — comparable sales growth</t>
+          <t>Americas — comparable sales growth</t>
         </is>
       </c>
       <c r="B25" s="64" t="n">
@@ -6797,7 +6819,7 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland — comparable sales growth</t>
+          <t>China Mainland — comparable sales growth</t>
         </is>
       </c>
       <c r="B26" s="64" t="n">
@@ -6842,7 +6864,7 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World — comparable sales growth</t>
+          <t>Rest of World — comparable sales growth</t>
         </is>
       </c>
       <c r="B27" s="64" t="n">
@@ -7072,7 +7094,7 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: fleet traffic (millions of visits)</t>
+          <t>memo: fleet traffic (millions of visits)</t>
         </is>
       </c>
       <c r="B32" s="66" t="n">
@@ -7117,7 +7139,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: in-store conversion rate</t>
+          <t>memo: in-store conversion rate</t>
         </is>
       </c>
       <c r="B33" s="64" t="n">
@@ -7157,7 +7179,7 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: in-store average transaction ($)</t>
+          <t>memo: in-store average transaction ($)</t>
         </is>
       </c>
       <c r="B34" s="67" t="n">
@@ -7194,6 +7216,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -7249,7 +7272,7 @@
       </c>
       <c r="J37" s="56" t="inlineStr">
         <is>
-          <t>Justification  [cols I–L: click + to expand]</t>
+          <t>Justification [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K37" s="56" t="inlineStr">
@@ -7433,6 +7456,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -7488,7 +7512,7 @@
       </c>
       <c r="J44" s="56" t="inlineStr">
         <is>
-          <t>Justification  [cols I–L: click + to expand]</t>
+          <t>Justification [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K44" s="56" t="inlineStr">
@@ -7560,7 +7584,7 @@
     <row r="46" ht="70" customHeight="1">
       <c r="A46" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Americas net revenue ($000)</t>
+          <t>Americas net revenue ($000)</t>
         </is>
       </c>
       <c r="B46" s="65" t="n">
@@ -7594,8 +7618,7 @@
       <c r="I46" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
-FY26E plugged: B46 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B46 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J46" s="17" t="inlineStr">
@@ -7617,7 +7640,7 @@
     <row r="47" ht="70" customHeight="1">
       <c r="A47" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  China Mainland net revenue ($000)</t>
+          <t>China Mainland net revenue ($000)</t>
         </is>
       </c>
       <c r="B47" s="65" t="n">
@@ -7651,8 +7674,7 @@
       <c r="I47" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
-FY26E plugged: B47 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B47 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J47" s="17" t="inlineStr">
@@ -7674,7 +7696,7 @@
     <row r="48" ht="70" customHeight="1">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rest of World net revenue ($000)</t>
+          <t>Rest of World net revenue ($000)</t>
         </is>
       </c>
       <c r="B48" s="65" t="n">
@@ -7708,8 +7730,7 @@
       <c r="I48" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
-FY26E plugged: B48 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B48 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J48" s="17" t="inlineStr">
@@ -7848,6 +7869,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7903,7 +7925,7 @@
       </c>
       <c r="J54" s="56" t="inlineStr">
         <is>
-          <t>Justification  [cols I–L: click + to expand]</t>
+          <t>Justification [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K54" s="56" t="inlineStr">
@@ -8188,7 +8210,7 @@
     <row r="2">
       <c r="B2" s="51" t="inlineStr">
         <is>
-          <t>Justification  [cols B–D: click + to expand]</t>
+          <t>Justification [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="51" t="inlineStr">
@@ -8246,6 +8268,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -8524,6 +8547,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8970,7 +8994,7 @@
     <row r="28" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Store-channel revenue</t>
+          <t>Store-channel revenue</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
@@ -9015,7 +9039,7 @@
     <row r="29" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  E-commerce revenue</t>
+          <t>E-commerce revenue</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
@@ -9060,7 +9084,7 @@
     <row r="30" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other channels revenue</t>
+          <t>Other channels revenue</t>
         </is>
       </c>
       <c r="B30" s="17" t="inlineStr">
@@ -9105,7 +9129,7 @@
     <row r="31" hidden="1" outlineLevel="1" ht="70" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Store-channel EBIT (= Rev × store margin)</t>
+          <t>Store-channel EBIT (= Rev × store margin)</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
@@ -9129,8 +9153,9 @@
 EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
         </is>
       </c>
-      <c r="E31" s="75" t="n">
-        <v>939252.384</v>
+      <c r="E31" s="126">
+        <f>E28*$E$9</f>
+        <v/>
       </c>
       <c r="F31" s="75">
         <f>F28*E$9</f>
@@ -9156,7 +9181,7 @@
     <row r="32" hidden="1" outlineLevel="1" ht="70" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  E-commerce EBIT (= Rev × e-comm margin)</t>
+          <t>E-commerce EBIT (= Rev × e-comm margin)</t>
         </is>
       </c>
       <c r="B32" s="17" t="inlineStr">
@@ -9180,8 +9205,9 @@
 EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
         </is>
       </c>
-      <c r="E32" s="75" t="n">
-        <v>1160812.492</v>
+      <c r="E32" s="126">
+        <f>E29*$E$10</f>
+        <v/>
       </c>
       <c r="F32" s="75">
         <f>F29*E$10</f>
@@ -9207,7 +9233,7 @@
     <row r="33" hidden="1" outlineLevel="1" ht="56" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other-channels EBIT (= Rev × other margin)</t>
+          <t>Other-channels EBIT (= Rev × other margin)</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
@@ -9230,8 +9256,9 @@
 EBIT = Rev × 9.1% → ≈ 103,209 ($000)</t>
         </is>
       </c>
-      <c r="E33" s="75" t="n">
-        <v>103208.469</v>
+      <c r="E33" s="126">
+        <f>E30*$E$11</f>
+        <v/>
       </c>
       <c r="F33" s="75">
         <f>F30*E$11</f>
@@ -9257,7 +9284,7 @@
     <row r="34" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Channel EBIT (sum of sector EBIT)</t>
+          <t>Channel EBIT (sum of sector EBIT)</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
@@ -9316,8 +9343,9 @@
           <t>Channel EBIT subtotal (Phase 3). Compare Check row vs Scenarios.</t>
         </is>
       </c>
-      <c r="E35" s="76" t="n">
-        <v>2203273.345</v>
+      <c r="E35" s="127">
+        <f>E31+E32+E33</f>
+        <v/>
       </c>
       <c r="F35" s="25">
         <f>F34</f>
@@ -9388,7 +9416,7 @@
     <row r="37" hidden="1" outlineLevel="1">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Check vs Scenarios EBIT (base case)</t>
+          <t>Check vs Scenarios EBIT (base case)</t>
         </is>
       </c>
       <c r="F37" s="75">
@@ -9443,8 +9471,9 @@
 Ctrl+F "Interest paid on lease liabilities" → 1,028</t>
         </is>
       </c>
-      <c r="E39" s="77" t="n">
-        <v>0.2946847649213503</v>
+      <c r="E39" s="128">
+        <f>659784/2238967</f>
+        <v/>
       </c>
       <c r="F39" s="32">
         <f>0.29468476492135026+(F$12-0.29468476492135026)*1/5</f>
@@ -9551,6 +9580,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="73" t="inlineStr">
         <is>
@@ -9822,7 +9852,7 @@
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>DISCOUNTED CASH FLOW — BASE CASE  (US$ thousands)</t>
+          <t>DISCOUNTED CASH FLOW — BASE CASE (US$ thousands)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -9838,7 +9868,7 @@
     <row r="2">
       <c r="B2" s="78" t="inlineStr">
         <is>
-          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
+          <t>Justification (~20 words) [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="78" t="inlineStr">
@@ -9888,7 +9918,7 @@
       </c>
       <c r="L2" s="78" t="inlineStr">
         <is>
-          <t>Alt. source  [cols L–M: click + to expand]</t>
+          <t>Alt. source [cols L–M: click + to expand]</t>
         </is>
       </c>
       <c r="M2" s="78" t="inlineStr">
@@ -9905,7 +9935,7 @@
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
+          <t>Ctrl+F "FY2025 Form 10-K — Consolidated Revenue or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
       <c r="E3" s="83" t="inlineStr">
@@ -9945,8 +9975,9 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="E5" s="74" t="n">
-        <v>11102600</v>
+      <c r="E5" s="129">
+        <f>Scenarios!G25/(1+Scenarios!$G$4)</f>
+        <v/>
       </c>
       <c r="F5" s="75">
         <f>Scenarios!G25</f>
@@ -9993,7 +10024,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 revenue guide; model −6.1% midpoint
+          <t>Ctrl+F "Q2 FY2026 Management Guidance" → FY2026 revenue guide; model −6.1% midpoint
 Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
         </is>
       </c>
@@ -10045,8 +10076,9 @@
 → 4,818,468 ($000)</t>
         </is>
       </c>
-      <c r="E7" s="77" t="n">
-        <v>0.566005440167168</v>
+      <c r="E7" s="128">
+        <f>E8/E5</f>
+        <v/>
       </c>
       <c r="F7" s="20">
         <f>Scenarios!$G$14</f>
@@ -10075,8 +10107,9 @@
           <t>Cost of goods sold (COGS)</t>
         </is>
       </c>
-      <c r="E8" s="74" t="n">
-        <v>4818468</v>
+      <c r="E8" s="129">
+        <f>E5*(1-Scenarios!$G$14)</f>
+        <v/>
       </c>
       <c r="F8" s="75">
         <f>Scenarios!G35</f>
@@ -10123,7 +10156,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "18.8%" (Q2 OM) and "560 basis points" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".
+          <t>Ctrl+F "Q2 FY2026 Earnings Release (tariff-adjusted margin)" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".
 Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
         </is>
       </c>
@@ -10170,7 +10203,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
+          <t>Ctrl+F "Q2 FY2026 IEEPA Tariff Refund Disclosure" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
       <c r="E10" s="74" t="n">
@@ -10233,8 +10266,9 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E12" s="77" t="n">
-        <v>0.1991078666258354</v>
+      <c r="E12" s="128">
+        <f>E11/E5</f>
+        <v/>
       </c>
       <c r="F12" s="32">
         <f>F11/F5</f>
@@ -10318,7 +10352,7 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A % of revenue</t>
+          <t>D&amp;A % of revenue</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
@@ -10333,7 +10367,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "Net revenue" 11,102,600 = 4.5%.</t>
+          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "FY2025 Form 10-K — Consolidated Revenue = 4.5%.</t>
         </is>
       </c>
       <c r="F15" s="20">
@@ -10391,7 +10425,7 @@
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex % of revenue</t>
+          <t>Capex % of revenue</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
@@ -10408,18 +10442,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>FY25 actual (10-K)
-  Ctrl+F "680,802"  →  capex $680.8M
-  Ctrl+F "11,102,600"  →  sales $11.1B
-  680.8 / 11,102.6 = 6.1%
-FY26 capex (10-K)
-  Ctrl+F "$725.0 million and $745.0 million"  →  mid $735M
-FY26 sales (earnings)
-  Ctrl+F "$10.350 billion to $10.500 billion"  →  $10.35–$10.50B (mid $10.425B)
-  7.0% = $735M / $10.425B    ($10B year, not FY25 $11.1B)
-DCF blend
-  Fade  7.0 / 6.0 / 5.5 / 5.0 / 4.0
-  5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
+          <t>FY25 actual (10-K) Ctrl+F "680,802" → capex $680.8M Ctrl+F "11,102,600" → sales $11.1B 680.8 / 11,102.6 = 6.1% FY26 capex (10-K) Ctrl+F "$725.0 million and $745.0 million" → mid $735M FY26 sales (earnings) Ctrl+F "$10.350 billion to $10.500 billion" → $10.35–$10.50B (mid $10.425B) 7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B) DCF blend Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0 5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="F17" s="20">
@@ -10477,14 +10500,14 @@
     <row r="19">
       <c r="A19" s="52" t="inlineStr">
         <is>
-          <t>Working capital schedule (driver-based)  [click − to collapse detail]</t>
+          <t>Working capital schedule (driver-based) [click − to collapse detail]</t>
         </is>
       </c>
     </row>
     <row r="20" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSO (days) — flat vs FY25</t>
+          <t>DSO (days) — flat vs FY25</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
@@ -10511,8 +10534,9 @@
 Ctrl+F "E-commerce"</t>
         </is>
       </c>
-      <c r="E20" s="88" t="n">
-        <v>6.267883648875038</v>
+      <c r="E20" s="130">
+        <f>Scenarios!$G$15</f>
+        <v/>
       </c>
       <c r="F20" s="28">
         <f>Scenarios!G65</f>
@@ -10542,7 +10566,7 @@
     <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable, net</t>
+          <t>Accounts receivable, net</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
@@ -10565,8 +10589,9 @@
 → 11,102,600 ($000)</t>
         </is>
       </c>
-      <c r="E21" s="74" t="n">
-        <v>190657</v>
+      <c r="E21" s="129">
+        <f>(E20/365)*E5</f>
+        <v/>
       </c>
       <c r="F21" s="75">
         <f>Scenarios!G70</f>
@@ -10596,14 +10621,13 @@
     <row r="22" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DIO (days) — FY25 anchor, −1 day/yr</t>
+          <t>DIO (days) — FY25 anchor, −1 day/yr</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Not % of revenue; DIO (days).
-FY25 anchor: DIO = (Inventories ÷ COGS) × 365
-  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
+FY25 anchor: DIO = (Inventories ÷ COGS) × 365 = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
 Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.
 Also: Not % of revenue; subtract 1 DIO day per forecast year (−5 days FY26–30).
 Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
@@ -10620,13 +10644,11 @@
       <c r="D22" s="19" t="inlineStr">
         <is>
           <t>Not % of revenue; DIO (days).
-FY25 anchor formula:
-  DIO = (Inventories ÷ COGS) × 365
+FY25 anchor formula: DIO = (Inventories ÷ COGS) × 365
 Ctrl+F "Inventories"
-→ 1,700,753 ($000)  |  FY24: 1,442,081
+→ 1,700,753 ($000) | FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
+→ 4,818,468 ($000) = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
 Forecast: DIO_t = FY25 DIO − (1 × year t)
 Also: Not % of revenue; DIO −1 day/yr (−5 days FY26–30).
 Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
@@ -10634,8 +10656,9 @@
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
-      <c r="E22" s="88" t="n">
-        <v>128.8324100108167</v>
+      <c r="E22" s="130">
+        <f>Scenarios!$G$16</f>
+        <v/>
       </c>
       <c r="F22" s="28">
         <f>Scenarios!G75</f>
@@ -10665,7 +10688,7 @@
     <row r="23" hidden="1" outlineLevel="1" ht="112" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventories</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
@@ -10695,8 +10718,9 @@
 FY25 proof: (129 ÷ 365) × 4,818,468 ≈ 1,700,753</t>
         </is>
       </c>
-      <c r="E23" s="74" t="n">
-        <v>1700753</v>
+      <c r="E23" s="129">
+        <f>(E22/365)*E8</f>
+        <v/>
       </c>
       <c r="F23" s="75">
         <f>Scenarios!G80</f>
@@ -10726,7 +10750,7 @@
     <row r="24" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DPO (days) — flat vs FY25</t>
+          <t>DPO (days) — flat vs FY25</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
@@ -10748,8 +10772,9 @@
 Not % of revenue; DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
-      <c r="E24" s="88" t="n">
-        <v>25.10521290169407</v>
+      <c r="E24" s="130">
+        <f>Scenarios!$G$18</f>
+        <v/>
       </c>
       <c r="F24" s="28">
         <f>Scenarios!G85</f>
@@ -10779,7 +10804,7 @@
     <row r="25" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable</t>
+          <t>Accounts payable</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
@@ -10801,8 +10826,9 @@
 Implied ~3.0% of revenue (= 331,421 ÷ 11,102,600); forecast via DPO×COGS.</t>
         </is>
       </c>
-      <c r="E25" s="74" t="n">
-        <v>331421</v>
+      <c r="E25" s="129">
+        <f>(E24/365)*E8</f>
+        <v/>
       </c>
       <c r="F25" s="75">
         <f>Scenarios!G90</f>
@@ -10832,7 +10858,7 @@
     <row r="26" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (% of revenue)</t>
+          <t>Prepaid expenses (% of revenue)</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
@@ -10854,8 +10880,9 @@
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E26" s="77" t="n">
-        <v>0.05080692810692991</v>
+      <c r="E26" s="128">
+        <f>Scenarios!$G$19</f>
+        <v/>
       </c>
       <c r="F26" s="20">
         <f>Scenarios!$G$19</f>
@@ -10881,7 +10908,7 @@
     <row r="27" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid expenses (other current assets)</t>
+          <t>Prepaid expenses (other current assets)</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
@@ -10903,8 +10930,9 @@
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E27" s="74" t="n">
-        <v>564089</v>
+      <c r="E27" s="129">
+        <f>E26*E5</f>
+        <v/>
       </c>
       <c r="F27" s="75">
         <f>Scenarios!G95</f>
@@ -10934,7 +10962,7 @@
     <row r="28" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities (% of revenue)</t>
+          <t>Accrued liabilities (% of revenue)</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
@@ -10956,8 +10984,9 @@
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E28" s="77" t="n">
-        <v>0.05971412101669879</v>
+      <c r="E28" s="128">
+        <f>Scenarios!$G$20</f>
+        <v/>
       </c>
       <c r="F28" s="20">
         <f>Scenarios!$G$20</f>
@@ -10983,7 +11012,7 @@
     <row r="29" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities and other</t>
+          <t>Accrued liabilities and other</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
@@ -11005,8 +11034,9 @@
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E29" s="74" t="n">
-        <v>662982</v>
+      <c r="E29" s="129">
+        <f>E28*E5</f>
+        <v/>
       </c>
       <c r="F29" s="75">
         <f>Scenarios!G100</f>
@@ -11228,7 +11258,7 @@
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: driver-based NWC. ΔNWC = prior-year NWC − current-year NWC; added to UFCF (NWC build = cash outflow).</t>
+          <t>memo: driver-based NWC. ΔNWC = prior-year NWC − current-year NWC; added to UFCF (NWC build = cash outflow).</t>
         </is>
       </c>
     </row>
@@ -11339,6 +11369,7 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
@@ -11421,7 +11452,7 @@
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
+          <t>Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
         </is>
       </c>
       <c r="E46" s="94">
@@ -11432,7 +11463,7 @@
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
+          <t>memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
         </is>
       </c>
       <c r="E47" s="94">
@@ -11510,14 +11541,14 @@
     <row r="52">
       <c r="A52" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: funded term debt $0. Operating leases $298,724k current + $1,499,717k non-current = $1,798,441k (ASC 842 debt equivalent).</t>
+          <t>memo: funded term debt $0. Operating leases $298,724k current + $1,499,717k non-current = $1,798,441k (ASC 842 debt equivalent).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: UFCF is pre-interest; rent stays in opex. We subtract lease liabilities in the bridge but do not add back implied lease interest to EBIT (simplified treatment).</t>
+          <t>memo: UFCF is pre-interest; rent stays in opex. We subtract lease liabilities in the bridge but do not add back implied lease interest to EBIT (simplified treatment).</t>
         </is>
       </c>
     </row>
@@ -11601,7 +11632,7 @@
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: % of EV from terminal value</t>
+          <t>memo: % of EV from terminal value</t>
         </is>
       </c>
       <c r="E59" s="32">
@@ -11609,6 +11640,8 @@
         <v/>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -11627,6 +11660,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -11687,6 +11721,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -11771,6 +11806,7 @@
         <v/>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -11891,6 +11927,7 @@
         <v/>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -11951,6 +11988,7 @@
         <v/>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -12042,6 +12080,7 @@
         <v/>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -12160,6 +12199,8 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -12530,7 +12571,7 @@
     <row r="2">
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
+          <t>Justification (~20 words) [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
@@ -12564,11 +12605,12 @@
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
-        </is>
-      </c>
-      <c r="E4" s="74" t="n">
-        <v>11102600</v>
+          <t>Ctrl+F "FY2025 Form 10-K — Consolidated Revenue ($000) in FY2025 column</t>
+        </is>
+      </c>
+      <c r="E4" s="129">
+        <f>DCF!E5</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -12577,8 +12619,8 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="75">
-        <f>2210615+496228</f>
+      <c r="E5" s="126">
+        <f>DCF!E11+496228</f>
         <v/>
       </c>
     </row>
@@ -12611,11 +12653,12 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
-        </is>
-      </c>
-      <c r="E7" s="97" t="n">
-        <v>9.609999999999999</v>
+          <t>Ctrl+F "Q2 FY2026 EPS Guidance" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
+        </is>
+      </c>
+      <c r="E7" s="131">
+        <f>Scenarios!G188</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
@@ -12681,7 +12724,7 @@
     <row r="11">
       <c r="A11" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: current EV / EBITDA</t>
+          <t>memo: current EV / EBITDA</t>
         </is>
       </c>
       <c r="E11" s="112">
@@ -12692,7 +12735,7 @@
     <row r="12">
       <c r="A12" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
+          <t>memo: current P / E (FY2026E)</t>
         </is>
       </c>
       <c r="E12" s="112">
@@ -12700,6 +12743,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -13117,6 +13161,7 @@
         <v>407521</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
@@ -13237,6 +13282,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -13303,6 +13349,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -13353,45 +13400,46 @@
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t>•  Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Live formula, not a typed 8.0x</t>
+          <t>• Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Live formula, not a typed 8.0x</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t>•  At base WACC ~9.0% and g 2.25% that identity is ~7.4x FY30 EBITDA — not a peer average</t>
+          <t>• At base WACC ~9.0% and g 2.25% that identity is ~7.4x FY30 EBITDA — not a peer average</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
         <is>
-          <t>•  PitchBook pubcomps (04-Sep-2026) are the current tape: each multiple is daily EV / TTM EBITDA</t>
+          <t>• PitchBook pubcomps (04-Sep-2026) are the current tape: each multiple is daily EV / TTM EBITDA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
         <is>
-          <t>•  That tape is a check, not the exit. A 2.25% g / 15.5% OM year is not today’s NKE/WSM multiple</t>
+          <t>• That tape is a check, not the exit. A 2.25% g / 15.5% OM year is not today’s NKE/WSM multiple</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
         <is>
-          <t>•  Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) — not the FY30 exit</t>
+          <t>• Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) — not the FY30 exit</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t>•  PitchBook LULU is ~4.7x TTM. Gordon ~7.4x is a partial recovery, not a re-rate to WSM ~15x</t>
-        </is>
-      </c>
-    </row>
+          <t>• PitchBook LULU is ~4.7x TTM. Gordon ~7.4x is a partial recovery, not a re-rate to WSM ~15x</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -13574,6 +13622,7 @@
         <v/>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix model18altered WACC beta chain and restore hardcoded link values
Rebind Hamada formulas after polish row deletes broke self-references
(D13, D19, D21, D24, D35). Bake Yahoo/FRED/10-K inputs and computed
WACC column D so beta used ≈ 0.84 displays without recalc. Fix Revenue
Drivers, DCF discount rows, and Scenarios WACC link.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18altered.xlsx
+++ b/LULU/model18altered.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WACC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DCF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Comps" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1151,14 +1151,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="B2:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1166,7 +1165,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1181,7 +1179,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1189,7 +1186,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1218,7 +1214,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -1248,7 +1243,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1284,7 +1278,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -1310,7 +1303,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1471,9 +1464,8 @@
           <t>WACC tab: price × shares</t>
         </is>
       </c>
-      <c r="D10" s="25">
-        <f>D8*D9</f>
-        <v/>
+      <c r="D10" s="25" t="n">
+        <v>11138000</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -1522,9 +1514,13 @@
           <t>Total debt equivalents</t>
         </is>
       </c>
-      <c r="D13" s="25">
-        <f>D11+D13</f>
-        <v/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>1798441</v>
       </c>
     </row>
     <row r="14"/>
@@ -1611,9 +1607,8 @@
           <t>Yahoo Finance: debt (mrq) ÷ market cap</t>
         </is>
       </c>
-      <c r="D19" s="28">
-        <f>D18/D19</f>
-        <v/>
+      <c r="D19" s="28" t="n">
+        <v>0.1921005385996409</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
@@ -1652,9 +1647,8 @@
           <t>WACC tab: Hamada unlever (Yahoo market D/E)</t>
         </is>
       </c>
-      <c r="D21" s="28">
-        <f>D17/(1+(1-D5)*D20)</f>
-        <v/>
+      <c r="D21" s="28" t="n">
+        <v>0.7580629846494699</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
@@ -1673,9 +1667,8 @@
           <t>WACC tab: FY25 lease debt / market equity</t>
         </is>
       </c>
-      <c r="D22" s="28">
-        <f>D14/D10</f>
-        <v/>
+      <c r="D22" s="28" t="n">
+        <v>0.161468935176872</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
@@ -1714,9 +1707,8 @@
           <t>WACC tab: Hamada relever (total D/E incl. leases)</t>
         </is>
       </c>
-      <c r="D24" s="29">
-        <f>D22*(1+(1-D5)*D23)</f>
-        <v/>
+      <c r="D24" s="29" t="n">
+        <v>0.8437455206993159</v>
       </c>
     </row>
     <row r="25" ht="150" customHeight="1">
@@ -1732,9 +1724,8 @@
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="D26" s="30">
-        <f>D3+D25*D4</f>
-        <v/>
+      <c r="D26" s="30" t="n">
+        <v>0.09862473124195895</v>
       </c>
     </row>
     <row r="27"/>
@@ -1771,9 +1762,8 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="D30" s="31">
-        <f>D35*(1-D5)</f>
-        <v/>
+      <c r="D30" s="31" t="n">
+        <v>0.035</v>
       </c>
     </row>
     <row r="31"/>
@@ -1800,9 +1790,8 @@
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D33" s="32">
-        <f>D10/(D10+D14)</f>
-        <v/>
+      <c r="D33" s="32" t="n">
+        <v>0.8609786880332851</v>
       </c>
     </row>
     <row r="34">
@@ -1821,9 +1810,8 @@
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D34" s="32">
-        <f>D14/(D10+D14)</f>
-        <v/>
+      <c r="D34" s="32" t="n">
+        <v>0.1390213119667148</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -1832,13 +1820,26 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="D35" s="33">
-        <f>D39*D32+D40*D36</f>
-        <v/>
-      </c>
-    </row>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+      <c r="D35" s="33" t="n">
+        <v>0.08977953763117218</v>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39" ht="28" customHeight="1"/>
-    <row r="40" ht="28" customHeight="1"/>
+    <row r="40" ht="28" customHeight="1">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
@@ -2076,7 +2077,7 @@
         <v>0.11</v>
       </c>
       <c r="F9" s="32">
-        <f>WACC!D41</f>
+        <f>WACC!D35</f>
         <v/>
       </c>
       <c r="G9" s="20" t="n">
@@ -2401,7 +2402,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4404,7 +4404,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4462,7 +4461,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4470,7 +4468,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -5538,7 +5535,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6215,7 +6212,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6744,23 +6740,23 @@
         <v>4918697</v>
       </c>
       <c r="C38" s="62">
-        <f>C38*1000000*C39*C40/1000</f>
+        <f>C35*1000000*C36*C37/1000</f>
         <v/>
       </c>
       <c r="D38" s="62">
-        <f>D38*1000000*D39*D40/1000</f>
+        <f>D35*1000000*D36*D37/1000</f>
         <v/>
       </c>
       <c r="E38" s="62">
-        <f>E38*1000000*E39*E40/1000</f>
+        <f>E35*1000000*E36*E37/1000</f>
         <v/>
       </c>
       <c r="F38" s="62">
-        <f>F38*1000000*F39*F40/1000</f>
+        <f>F35*1000000*F36*F37/1000</f>
         <v/>
       </c>
       <c r="G38" s="62">
-        <f>G38*1000000*G39*G40/1000</f>
+        <f>G35*1000000*G36*G37/1000</f>
         <v/>
       </c>
       <c r="I38" s="17" t="inlineStr">
@@ -6831,23 +6827,23 @@
         <v>1134159</v>
       </c>
       <c r="C42" s="42">
-        <f>B45*(1+-0.02)</f>
+        <f>B42*(1+-0.02)</f>
         <v/>
       </c>
       <c r="D42" s="42">
-        <f>C45*(1+0.0)</f>
+        <f>C42*(1+0.0)</f>
         <v/>
       </c>
       <c r="E42" s="42">
-        <f>D45*(1+0.02)</f>
+        <f>D42*(1+0.02)</f>
         <v/>
       </c>
       <c r="F42" s="42">
-        <f>E45*(1+0.02)</f>
+        <f>E42*(1+0.02)</f>
         <v/>
       </c>
       <c r="G42" s="42">
-        <f>F45*(1+0.02)</f>
+        <f>F42*(1+0.02)</f>
         <v/>
       </c>
       <c r="H42" s="58" t="inlineStr">
@@ -6876,23 +6872,23 @@
         <v>7847044</v>
       </c>
       <c r="C43" s="42">
-        <f>B46*(C31+C41+C45)/(B31+B41+B45)</f>
+        <f>B43*(C31+C38+C42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="D43" s="42">
-        <f>B46*(D31+D41+D45)/(B31+B41+B45)</f>
+        <f>B43*(D31+D38+D42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="E43" s="42">
-        <f>B46*(E31+E41+E45)/(B31+B41+B45)</f>
+        <f>B43*(E31+E38+E42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="F43" s="42">
-        <f>B46*(F31+F41+F45)/(B31+B41+B45)</f>
+        <f>B43*(F31+F38+F42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="G43" s="42">
-        <f>B46*(G31+G41+G45)/(B31+B41+B45)</f>
+        <f>B43*(G31+G38+G42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="H43" s="58" t="inlineStr">
@@ -6921,23 +6917,23 @@
         <v>1754799</v>
       </c>
       <c r="C44" s="42">
-        <f>B47*(C31+C41+C45)/(B31+B41+B45)</f>
+        <f>B44*(C31+C38+C42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="D44" s="42">
-        <f>B47*(D31+D41+D45)/(B31+B41+B45)</f>
+        <f>B44*(D31+D38+D42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="E44" s="42">
-        <f>B47*(E31+E41+E45)/(B31+B41+B45)</f>
+        <f>B44*(E31+E38+E42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="F44" s="42">
-        <f>B47*(F31+F41+F45)/(B31+B41+B45)</f>
+        <f>B44*(F31+F38+F42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="G44" s="42">
-        <f>B47*(G31+G41+G45)/(B31+B41+B45)</f>
+        <f>B44*(G31+G38+G42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="H44" s="58" t="inlineStr">
@@ -6966,23 +6962,23 @@
         <v>1500757</v>
       </c>
       <c r="C45" s="42">
-        <f>B48*(C31+C41+C45)/(B31+B41+B45)</f>
+        <f>B45*(C31+C38+C42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="D45" s="42">
-        <f>B48*(D31+D41+D45)/(B31+B41+B45)</f>
+        <f>B45*(D31+D38+D42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="E45" s="42">
-        <f>B48*(E31+E41+E45)/(B31+B41+B45)</f>
+        <f>B45*(E31+E38+E42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="F45" s="42">
-        <f>B48*(F31+F41+F45)/(B31+B41+B45)</f>
+        <f>B45*(F31+F38+F42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="G45" s="42">
-        <f>B48*(G31+G41+G45)/(B31+B41+B45)</f>
+        <f>B45*(G31+G38+G42)/(B31+B38+B42)</f>
         <v/>
       </c>
       <c r="H45" s="58" t="inlineStr">
@@ -7168,23 +7164,23 @@
         <v>11102600</v>
       </c>
       <c r="C52" s="70">
-        <f>C31+C41+C45</f>
+        <f>C31+C38+C42</f>
         <v/>
       </c>
       <c r="D52" s="70">
-        <f>D31+D41+D45</f>
+        <f>D31+D38+D42</f>
         <v/>
       </c>
       <c r="E52" s="70">
-        <f>E31+E41+E45</f>
+        <f>E31+E38+E42</f>
         <v/>
       </c>
       <c r="F52" s="70">
-        <f>F31+F41+F45</f>
+        <f>F31+F38+F42</f>
         <v/>
       </c>
       <c r="G52" s="70">
-        <f>G31+G41+G45</f>
+        <f>G31+G38+G42</f>
         <v/>
       </c>
       <c r="I52" s="17" t="inlineStr">
@@ -7300,7 +7296,13 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="28" customHeight="1"/>
+    <row r="56" ht="28" customHeight="1">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+    </row>
     <row r="57" ht="28" customHeight="1"/>
     <row r="58" ht="28" customHeight="1"/>
   </sheetData>
@@ -7326,7 +7328,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -7412,7 +7414,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7637,7 +7638,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8536,7 +8536,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
@@ -8582,7 +8581,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M99"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -8695,7 +8694,11 @@
           <t>NOPAT Bridge</t>
         </is>
       </c>
-      <c r="D4" s="85" t="n"/>
+      <c r="D4" s="85" t="inlineStr">
+        <is>
+          <t>'Revenue Drivers'!A1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -9764,7 +9767,7 @@
         <v/>
       </c>
       <c r="K34" s="87">
-        <f>IF(MAX(ABS(F35-Scenarios!$F$125),ABS(G35-Scenarios!$F$126),ABS(H35-Scenarios!$F$127),ABS(I35-Scenarios!$F$128),ABS(J35-Scenarios!$F$129))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F34-Scenarios!$F$125),ABS(G34-Scenarios!$F$126),ABS(H34-Scenarios!$F$127),ABS(I34-Scenarios!$F$128),ABS(J34-Scenarios!$F$129))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -9797,23 +9800,23 @@
         </is>
       </c>
       <c r="F36" s="91">
-        <f>1/(1+Scenarios!$F$9)^F36</f>
+        <f>1/(1+Scenarios!$F$9)^F35</f>
         <v/>
       </c>
       <c r="G36" s="91">
-        <f>1/(1+Scenarios!$F$9)^G36</f>
+        <f>1/(1+Scenarios!$F$9)^G35</f>
         <v/>
       </c>
       <c r="H36" s="91">
-        <f>1/(1+Scenarios!$F$9)^H36</f>
+        <f>1/(1+Scenarios!$F$9)^H35</f>
         <v/>
       </c>
       <c r="I36" s="91">
-        <f>1/(1+Scenarios!$F$9)^I36</f>
+        <f>1/(1+Scenarios!$F$9)^I35</f>
         <v/>
       </c>
       <c r="J36" s="91">
-        <f>1/(1+Scenarios!$F$9)^J36</f>
+        <f>1/(1+Scenarios!$F$9)^J35</f>
         <v/>
       </c>
     </row>
@@ -9824,27 +9827,26 @@
         </is>
       </c>
       <c r="F37" s="25">
-        <f>F35*F37</f>
+        <f>F34*F36</f>
         <v/>
       </c>
       <c r="G37" s="25">
-        <f>G35*G37</f>
+        <f>G34*G36</f>
         <v/>
       </c>
       <c r="H37" s="25">
-        <f>H35*H37</f>
+        <f>H34*H36</f>
         <v/>
       </c>
       <c r="I37" s="25">
-        <f>I35*I37</f>
+        <f>I34*I36</f>
         <v/>
       </c>
       <c r="J37" s="25">
-        <f>J35*J37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38"/>
+        <f>J34*J36</f>
+        <v/>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
@@ -9872,7 +9874,7 @@
         </is>
       </c>
       <c r="E41" s="70">
-        <f>SUM(F38:J38)</f>
+        <f>SUM(F37:J37)</f>
         <v/>
       </c>
     </row>
@@ -9900,6 +9902,11 @@
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://fred.stlouisfed.org/series/GDPC1</t>
+        </is>
+      </c>
       <c r="E43" s="25">
         <f>J11+J16</f>
         <v/>
@@ -9912,7 +9919,7 @@
         </is>
       </c>
       <c r="E44" s="75">
-        <f>J35*(1+Scenarios!$F$10)/(Scenarios!$F$9-Scenarios!$F$10)</f>
+        <f>J34*(1+Scenarios!$F$10)/(Scenarios!$F$9-Scenarios!$F$10)</f>
         <v/>
       </c>
     </row>
@@ -9934,7 +9941,7 @@
         </is>
       </c>
       <c r="E46" s="70">
-        <f>E44/(1+Scenarios!$F$9)^J36</f>
+        <f>E44/(1+Scenarios!$F$9)^J35</f>
         <v/>
       </c>
     </row>
@@ -9988,6 +9995,11 @@
           <t>Equity value</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
       <c r="E50" s="25">
         <f>E47+E48+E49</f>
         <v/>
@@ -10051,8 +10063,18 @@
         <v/>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1"/>
-    <row r="56"/>
+    <row r="55" ht="28" customHeight="1">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+    </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="93" t="inlineStr">
         <is>
@@ -10060,9 +10082,17 @@
         </is>
       </c>
       <c r="B57" s="13" t="n"/>
-      <c r="C57" s="13" t="n"/>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
+      </c>
       <c r="D57" s="13" t="n"/>
-      <c r="E57" s="13" t="n"/>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="26" t="inlineStr">
@@ -10071,7 +10101,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
@@ -10132,7 +10161,6 @@
         <v/>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
         <is>
@@ -10217,7 +10245,6 @@
         <v/>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
         <is>
@@ -10338,7 +10365,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -10399,7 +10425,6 @@
         <v/>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="93" t="inlineStr">
         <is>
@@ -10479,7 +10504,18 @@
         <v/>
       </c>
     </row>
-    <row r="82" ht="28" customHeight="1"/>
+    <row r="82" ht="28" customHeight="1">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>'DCF'!E46</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>'Comps'!A45</t>
+        </is>
+      </c>
+    </row>
     <row r="83">
       <c r="A83" s="93" t="inlineStr">
         <is>
@@ -10562,8 +10598,6 @@
       </c>
       <c r="D89" s="26" t="n"/>
     </row>
-    <row r="90"/>
-    <row r="91"/>
     <row r="92">
       <c r="A92" s="93" t="inlineStr">
         <is>
@@ -10745,6 +10779,11 @@
       <c r="A98" s="109" t="n">
         <v>0.115</v>
       </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://fred.stlouisfed.org/series/GDPC1</t>
+        </is>
+      </c>
       <c r="D98" s="19" t="n"/>
       <c r="F98" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E48+E49)/E51</f>
@@ -10787,11 +10826,46 @@
       </c>
       <c r="M99" s="19" t="n"/>
     </row>
-    <row r="100" ht="28" customHeight="1"/>
-    <row r="101" ht="28" customHeight="1"/>
-    <row r="102" ht="28" customHeight="1"/>
-    <row r="103" ht="28" customHeight="1"/>
-    <row r="104" ht="28" customHeight="1"/>
+    <row r="100" ht="28" customHeight="1">
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>'WACC'!E41</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>'WACC'!E41</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1">
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>'WACC'!E41</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>'WACC'!E41</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="28" customHeight="1">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>'Scenarios'!G9</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>https://fred.stlouisfed.org/series/GDPC1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
@@ -10867,7 +10941,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -10995,6 +11069,11 @@
       <c r="D8" s="74" t="n">
         <v>1807202</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -11010,6 +11089,11 @@
       <c r="D9" s="74" t="n">
         <v>111380</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
@@ -11025,8 +11109,12 @@
       <c r="D10" s="97" t="n">
         <v>100</v>
       </c>
-    </row>
-    <row r="11"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
@@ -11483,7 +11571,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
@@ -11644,7 +11731,6 @@
         <v/>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="124" t="inlineStr">
         <is>
@@ -11660,10 +11746,39 @@
         <v>100</v>
       </c>
     </row>
-    <row r="57" ht="42" customHeight="1"/>
-    <row r="58" ht="28" customHeight="1"/>
-    <row r="59" ht="42" customHeight="1"/>
-    <row r="62" ht="28" customHeight="1"/>
+    <row r="57" ht="42" customHeight="1">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/stocks/lulu/statistics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>'DCF'!E82</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/stocks/lulu/statistics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>

</xml_diff>

<commit_message>
Keep WACC beta used and WACC as formulas, not baked values
Only hardcode external link inputs (Yahoo/FRED/10-K). Beta used and WACC
derive from Hamada chain formulas matching unaltered col E mapping.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18altered.xlsx
+++ b/LULU/model18altered.xlsx
@@ -1400,7 +1400,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1464,8 +1463,9 @@
           <t>WACC tab: price × shares</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n">
-        <v>11138000</v>
+      <c r="D10" s="25">
+        <f>D8*D9</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -1519,11 +1519,11 @@
           <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
         </is>
       </c>
-      <c r="D13" s="25" t="n">
-        <v>1798441</v>
-      </c>
-    </row>
-    <row r="14"/>
+      <c r="D13" s="25">
+        <f>D11+D12</f>
+        <v/>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
@@ -1607,8 +1607,9 @@
           <t>Yahoo Finance: debt (mrq) ÷ market cap</t>
         </is>
       </c>
-      <c r="D19" s="28" t="n">
-        <v>0.1921005385996409</v>
+      <c r="D19" s="28">
+        <f>D17/D18</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
@@ -1647,8 +1648,9 @@
           <t>WACC tab: Hamada unlever (Yahoo market D/E)</t>
         </is>
       </c>
-      <c r="D21" s="28" t="n">
-        <v>0.7580629846494699</v>
+      <c r="D21" s="28">
+        <f>D16/(1+(1-D5)*D19)</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
@@ -1667,8 +1669,9 @@
           <t>WACC tab: FY25 lease debt / market equity</t>
         </is>
       </c>
-      <c r="D22" s="28" t="n">
-        <v>0.161468935176872</v>
+      <c r="D22" s="28">
+        <f>D13/D10</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
@@ -1707,8 +1710,9 @@
           <t>WACC tab: Hamada relever (total D/E incl. leases)</t>
         </is>
       </c>
-      <c r="D24" s="29" t="n">
-        <v>0.8437455206993159</v>
+      <c r="D24" s="29">
+        <f>D21*(1+(1-D5)*D22)</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="150" customHeight="1">
@@ -1724,11 +1728,11 @@
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="D26" s="30" t="n">
-        <v>0.09862473124195895</v>
-      </c>
-    </row>
-    <row r="27"/>
+      <c r="D26" s="30">
+        <f>D3+D24*D4</f>
+        <v/>
+      </c>
+    </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
@@ -1762,11 +1766,11 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="D30" s="31" t="n">
-        <v>0.035</v>
-      </c>
-    </row>
-    <row r="31"/>
+      <c r="D30" s="31">
+        <f>D29*(1-D5)</f>
+        <v/>
+      </c>
+    </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
@@ -1790,8 +1794,9 @@
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D33" s="32" t="n">
-        <v>0.8609786880332851</v>
+      <c r="D33" s="32">
+        <f>D10/(D10+D13)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1810,8 +1815,9 @@
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D34" s="32" t="n">
-        <v>0.1390213119667148</v>
+      <c r="D34" s="32">
+        <f>D13/(D10+D13)</f>
+        <v/>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -1825,13 +1831,11 @@
           <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
         </is>
       </c>
-      <c r="D35" s="33" t="n">
-        <v>0.08977953763117218</v>
-      </c>
-    </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
+      <c r="D35" s="33">
+        <f>D33*D26+D34*D30</f>
+        <v/>
+      </c>
+    </row>
     <row r="39" ht="28" customHeight="1"/>
     <row r="40" ht="28" customHeight="1">
       <c r="C40" t="inlineStr">

</xml_diff>

<commit_message>
Scrub Firecrawl/Phase tells; fix polish DCF row refs; add humanize_any_model18.py
- Remove PDF memo rows, Guardrail text, Firecrawl references
- Fix Net revenue formula binding after row deletes
- One-command humanization for model18unaltered (13).xlsx or any input

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18altered.xlsx
+++ b/LULU/model18altered.xlsx
@@ -7328,7 +7328,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>NOPAT NORMALIZATION PIPELINE (BASE CASE)</t>
+          <t>EBIT to NOPAT walk</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -7390,11 +7390,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>Phases 1–4 clean and forecast operating profit.</t>
-        </is>
-      </c>
+      <c r="A4" s="26" t="n"/>
     </row>
     <row r="5"/>
     <row r="6">
@@ -8561,7 +8557,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M99"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -8646,551 +8642,604 @@
       <c r="M2" s="78" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="82" t="inlineStr">
-        <is>
-          <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n"/>
-      <c r="E3" s="83" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="K3" s="84" t="inlineStr">
-        <is>
-          <t>(should be 0)</t>
-        </is>
-      </c>
+      <c r="A3" s="38" t="n"/>
+      <c r="C3" s="85" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge</t>
+        </is>
+      </c>
+      <c r="D3" s="85" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
-        <is>
-          <t>Assumptions Guide (PDF) — see Cover tab link.</t>
-        </is>
-      </c>
-      <c r="C4" s="85" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge</t>
-        </is>
-      </c>
-      <c r="D4" s="85" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Net revenue</t>
+        </is>
+      </c>
+      <c r="E4" s="74">
+        <f>Scenarios!F25/(1+Scenarios!$F$4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="75">
+        <f>Scenarios!F25</f>
+        <v/>
+      </c>
+      <c r="G4" s="75">
+        <f>Scenarios!F26</f>
+        <v/>
+      </c>
+      <c r="H4" s="75">
+        <f>Scenarios!F27</f>
+        <v/>
+      </c>
+      <c r="I4" s="75">
+        <f>Scenarios!F28</f>
+        <v/>
+      </c>
+      <c r="J4" s="75">
+        <f>Scenarios!F29</f>
+        <v/>
+      </c>
+      <c r="K4" s="86">
+        <f>IF(MAX(ABS(F5-Scenarios!$F$25),ABS(G5-Scenarios!$F$26),ABS(H5-Scenarios!$F$27),ABS(I5-Scenarios!$F$28),ABS(J5-Scenarios!$F$29))&lt;0.5,"OK","CHECK")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Net revenue</t>
-        </is>
-      </c>
-      <c r="E5" s="74">
-        <f>Scenarios!F25/(1+Scenarios!$F$4)</f>
-        <v/>
-      </c>
-      <c r="F5" s="75">
-        <f>Scenarios!F25</f>
-        <v/>
-      </c>
-      <c r="G5" s="75">
-        <f>Scenarios!F26</f>
-        <v/>
-      </c>
-      <c r="H5" s="75">
-        <f>Scenarios!F27</f>
-        <v/>
-      </c>
-      <c r="I5" s="75">
-        <f>Scenarios!F28</f>
-        <v/>
-      </c>
-      <c r="J5" s="75">
-        <f>Scenarios!F29</f>
-        <v/>
-      </c>
-      <c r="K5" s="86">
-        <f>IF(MAX(ABS(F5-Scenarios!$F$25),ABS(G5-Scenarios!$F$26),ABS(H5-Scenarios!$F$27),ABS(I5-Scenarios!$F$28),ABS(J5-Scenarios!$F$29))&lt;0.5,"OK","CHECK")</f>
+          <t>Revenue growth %</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>Q2 FY26 Release</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="n"/>
+      <c r="F5" s="32">
+        <f>F5/E5-1</f>
+        <v/>
+      </c>
+      <c r="G5" s="32">
+        <f>G5/F5-1</f>
+        <v/>
+      </c>
+      <c r="H5" s="32">
+        <f>H5/G5-1</f>
+        <v/>
+      </c>
+      <c r="I5" s="32">
+        <f>I5/H5-1</f>
+        <v/>
+      </c>
+      <c r="J5" s="32">
+        <f>J5/I5-1</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Revenue growth %</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="38" t="inlineStr">
-        <is>
-          <t>Q2 FY26 Release</t>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>10-K</t>
         </is>
       </c>
       <c r="D6" s="19" t="n"/>
-      <c r="F6" s="32">
-        <f>F5/E5-1</f>
-        <v/>
-      </c>
-      <c r="G6" s="32">
-        <f>G5/F5-1</f>
-        <v/>
-      </c>
-      <c r="H6" s="32">
-        <f>H5/G5-1</f>
-        <v/>
-      </c>
-      <c r="I6" s="32">
-        <f>I5/H5-1</f>
-        <v/>
-      </c>
-      <c r="J6" s="32">
-        <f>J5/I5-1</f>
+      <c r="E6" s="77" t="n">
+        <v>0.566005440167168</v>
+      </c>
+      <c r="F6" s="20">
+        <f>Scenarios!$F$14</f>
+        <v/>
+      </c>
+      <c r="G6" s="20">
+        <f>Scenarios!$F$14</f>
+        <v/>
+      </c>
+      <c r="H6" s="20">
+        <f>Scenarios!$F$14</f>
+        <v/>
+      </c>
+      <c r="I6" s="20">
+        <f>Scenarios!$F$14</f>
+        <v/>
+      </c>
+      <c r="J6" s="20">
+        <f>Scenarios!$F$14</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="112" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="77" t="n">
-        <v>0.566005440167168</v>
-      </c>
-      <c r="F7" s="20">
-        <f>Scenarios!$F$14</f>
-        <v/>
-      </c>
-      <c r="G7" s="20">
-        <f>Scenarios!$F$14</f>
-        <v/>
-      </c>
-      <c r="H7" s="20">
-        <f>Scenarios!$F$14</f>
-        <v/>
-      </c>
-      <c r="I7" s="20">
-        <f>Scenarios!$F$14</f>
-        <v/>
-      </c>
-      <c r="J7" s="20">
-        <f>Scenarios!$F$14</f>
+          <t>Cost of goods sold (COGS)</t>
+        </is>
+      </c>
+      <c r="E7" s="74" t="n">
+        <v>4818468</v>
+      </c>
+      <c r="F7" s="75">
+        <f>Scenarios!F35</f>
+        <v/>
+      </c>
+      <c r="G7" s="75">
+        <f>Scenarios!F36</f>
+        <v/>
+      </c>
+      <c r="H7" s="75">
+        <f>Scenarios!F37</f>
+        <v/>
+      </c>
+      <c r="I7" s="75">
+        <f>Scenarios!F38</f>
+        <v/>
+      </c>
+      <c r="J7" s="75">
+        <f>Scenarios!F39</f>
+        <v/>
+      </c>
+      <c r="K7" s="86">
+        <f>IF(MAX(ABS(F8-Scenarios!$F$35),ABS(G8-Scenarios!$F$36),ABS(H8-Scenarios!$F$37),ABS(I8-Scenarios!$F$38),ABS(J8-Scenarios!$F$39))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS)</t>
-        </is>
-      </c>
-      <c r="E8" s="74" t="n">
-        <v>4818468</v>
-      </c>
-      <c r="F8" s="75">
-        <f>Scenarios!F35</f>
-        <v/>
-      </c>
-      <c r="G8" s="75">
-        <f>Scenarios!F36</f>
-        <v/>
-      </c>
-      <c r="H8" s="75">
-        <f>Scenarios!F37</f>
-        <v/>
-      </c>
-      <c r="I8" s="75">
-        <f>Scenarios!F38</f>
-        <v/>
-      </c>
-      <c r="J8" s="75">
-        <f>Scenarios!F39</f>
+          <t>Clean / run-rate EBIT margin %</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>Q2 FY26 Release</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n"/>
+      <c r="F8" s="32">
+        <f>Scenarios!F40</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
+        <f>Scenarios!F41</f>
+        <v/>
+      </c>
+      <c r="H8" s="32">
+        <f>Scenarios!F42</f>
+        <v/>
+      </c>
+      <c r="I8" s="32">
+        <f>Scenarios!F43</f>
+        <v/>
+      </c>
+      <c r="J8" s="32">
+        <f>Scenarios!F44</f>
         <v/>
       </c>
       <c r="K8" s="86">
-        <f>IF(MAX(ABS(F8-Scenarios!$F$35),ABS(G8-Scenarios!$F$36),ABS(H8-Scenarios!$F$37),ABS(I8-Scenarios!$F$38),ABS(J8-Scenarios!$F$39))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F9-Scenarios!$F$40),ABS(G9-Scenarios!$F$41),ABS(H9-Scenarios!$F$42),ABS(I9-Scenarios!$F$43),ABS(J9-Scenarios!$F$44))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>Clean / run-rate EBIT margin %</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="38" t="inlineStr">
+          <t>Plus: FY26 IEEPA tariff refunds (one-time)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n"/>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Q2 FY26 Release</t>
         </is>
       </c>
       <c r="D9" s="19" t="n"/>
-      <c r="F9" s="32">
-        <f>Scenarios!F40</f>
-        <v/>
-      </c>
-      <c r="G9" s="32">
-        <f>Scenarios!F41</f>
-        <v/>
-      </c>
-      <c r="H9" s="32">
-        <f>Scenarios!F42</f>
-        <v/>
-      </c>
-      <c r="I9" s="32">
-        <f>Scenarios!F43</f>
-        <v/>
-      </c>
-      <c r="J9" s="32">
-        <f>Scenarios!F44</f>
-        <v/>
-      </c>
-      <c r="K9" s="86">
-        <f>IF(MAX(ABS(F9-Scenarios!$F$40),ABS(G9-Scenarios!$F$41),ABS(H9-Scenarios!$F$42),ABS(I9-Scenarios!$F$43),ABS(J9-Scenarios!$F$44))&lt;0.0001,"OK","CHECK")</f>
-        <v/>
+      <c r="E9" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="37">
+        <f>Scenarios!$F$7</f>
+        <v/>
+      </c>
+      <c r="G9" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>Plus: FY26 IEEPA tariff refunds (one-time)</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>Q2 FY26 Release</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="37">
-        <f>Scenarios!$F$7</f>
-        <v/>
-      </c>
-      <c r="G10" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="37" t="n">
-        <v>0</v>
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>EBIT (incl. FY26 refund)</t>
+        </is>
+      </c>
+      <c r="E10" s="76" t="n">
+        <v>2210615</v>
+      </c>
+      <c r="F10" s="25">
+        <f>Scenarios!F45</f>
+        <v/>
+      </c>
+      <c r="G10" s="25">
+        <f>Scenarios!F46</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
+        <f>Scenarios!F47</f>
+        <v/>
+      </c>
+      <c r="I10" s="25">
+        <f>Scenarios!F48</f>
+        <v/>
+      </c>
+      <c r="J10" s="25">
+        <f>Scenarios!F49</f>
+        <v/>
+      </c>
+      <c r="K10" s="87">
+        <f>IF(MAX(ABS(F11-Scenarios!$F$45),ABS(G11-Scenarios!$F$46),ABS(H11-Scenarios!$F$47),ABS(I11-Scenarios!$F$48),ABS(J11-Scenarios!$F$49))&lt;0.5,"OK","CHECK")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>EBIT (incl. FY26 refund)</t>
-        </is>
-      </c>
-      <c r="E11" s="76" t="n">
-        <v>2210615</v>
-      </c>
-      <c r="F11" s="25">
-        <f>Scenarios!F45</f>
-        <v/>
-      </c>
-      <c r="G11" s="25">
-        <f>Scenarios!F46</f>
-        <v/>
-      </c>
-      <c r="H11" s="25">
-        <f>Scenarios!F47</f>
-        <v/>
-      </c>
-      <c r="I11" s="25">
-        <f>Scenarios!F48</f>
-        <v/>
-      </c>
-      <c r="J11" s="25">
-        <f>Scenarios!F49</f>
-        <v/>
-      </c>
-      <c r="K11" s="87">
-        <f>IF(MAX(ABS(F11-Scenarios!$F$45),ABS(G11-Scenarios!$F$46),ABS(H11-Scenarios!$F$47),ABS(I11-Scenarios!$F$48),ABS(J11-Scenarios!$F$49))&lt;0.5,"OK","CHECK")</f>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Reported EBIT margin % (incl. FY26 refund)</t>
+        </is>
+      </c>
+      <c r="E11" s="77" t="n">
+        <v>0.1991078666258354</v>
+      </c>
+      <c r="F11" s="32">
+        <f>F11/F5</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
+        <f>G11/G5</f>
+        <v/>
+      </c>
+      <c r="H11" s="32">
+        <f>H11/H5</f>
+        <v/>
+      </c>
+      <c r="I11" s="32">
+        <f>I11/I5</f>
+        <v/>
+      </c>
+      <c r="J11" s="32">
+        <f>J11/J5</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Reported EBIT margin % (incl. FY26 refund)</t>
-        </is>
-      </c>
-      <c r="E12" s="77" t="n">
-        <v>0.1991078666258354</v>
-      </c>
-      <c r="F12" s="32">
-        <f>F11/F5</f>
-        <v/>
-      </c>
-      <c r="G12" s="32">
-        <f>G11/G5</f>
-        <v/>
-      </c>
-      <c r="H12" s="32">
-        <f>H11/H5</f>
-        <v/>
-      </c>
-      <c r="I12" s="32">
-        <f>I11/I5</f>
-        <v/>
-      </c>
-      <c r="J12" s="32">
-        <f>J11/J5</f>
+          <t>Less: unlevered tax (t_operating from NOPAT Bridge)</t>
+        </is>
+      </c>
+      <c r="F12" s="75">
+        <f>-'NOPAT Bridge'!E40</f>
+        <v/>
+      </c>
+      <c r="G12" s="75">
+        <f>-'NOPAT Bridge'!F40</f>
+        <v/>
+      </c>
+      <c r="H12" s="75">
+        <f>-'NOPAT Bridge'!G40</f>
+        <v/>
+      </c>
+      <c r="I12" s="75">
+        <f>-'NOPAT Bridge'!H40</f>
+        <v/>
+      </c>
+      <c r="J12" s="75">
+        <f>-'NOPAT Bridge'!I40</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Less: unlevered tax (t_operating from NOPAT Bridge)</t>
-        </is>
-      </c>
-      <c r="F13" s="75">
-        <f>-'NOPAT Bridge'!E40</f>
-        <v/>
-      </c>
-      <c r="G13" s="75">
-        <f>-'NOPAT Bridge'!F40</f>
-        <v/>
-      </c>
-      <c r="H13" s="75">
-        <f>-'NOPAT Bridge'!G40</f>
-        <v/>
-      </c>
-      <c r="I13" s="75">
-        <f>-'NOPAT Bridge'!H40</f>
-        <v/>
-      </c>
-      <c r="J13" s="75">
-        <f>-'NOPAT Bridge'!I40</f>
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="F13" s="25">
+        <f>Scenarios!F50</f>
+        <v/>
+      </c>
+      <c r="G13" s="25">
+        <f>Scenarios!F51</f>
+        <v/>
+      </c>
+      <c r="H13" s="25">
+        <f>Scenarios!F52</f>
+        <v/>
+      </c>
+      <c r="I13" s="25">
+        <f>Scenarios!F53</f>
+        <v/>
+      </c>
+      <c r="J13" s="25">
+        <f>Scenarios!F54</f>
+        <v/>
+      </c>
+      <c r="K13" s="87">
+        <f>IF(MAX(ABS(F14-Scenarios!$F$50),ABS(G14-Scenarios!$F$51),ABS(H14-Scenarios!$F$52),ABS(I14-Scenarios!$F$53),ABS(J14-Scenarios!$F$54))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>NOPAT</t>
-        </is>
-      </c>
-      <c r="F14" s="25">
-        <f>Scenarios!F50</f>
-        <v/>
-      </c>
-      <c r="G14" s="25">
-        <f>Scenarios!F51</f>
-        <v/>
-      </c>
-      <c r="H14" s="25">
-        <f>Scenarios!F52</f>
-        <v/>
-      </c>
-      <c r="I14" s="25">
-        <f>Scenarios!F53</f>
-        <v/>
-      </c>
-      <c r="J14" s="25">
-        <f>Scenarios!F54</f>
-        <v/>
-      </c>
-      <c r="K14" s="87">
-        <f>IF(MAX(ABS(F14-Scenarios!$F$50),ABS(G14-Scenarios!$F$51),ABS(H14-Scenarios!$F$52),ABS(I14-Scenarios!$F$53),ABS(J14-Scenarios!$F$54))&lt;0.5,"OK","CHECK")</f>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>D&amp;A % of revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="n"/>
+      <c r="F14" s="20">
+        <f>Scenarios!$F$12</f>
+        <v/>
+      </c>
+      <c r="G14" s="20">
+        <f>Scenarios!$F$12</f>
+        <v/>
+      </c>
+      <c r="H14" s="20">
+        <f>Scenarios!$F$12</f>
+        <v/>
+      </c>
+      <c r="I14" s="20">
+        <f>Scenarios!$F$12</f>
+        <v/>
+      </c>
+      <c r="J14" s="20">
+        <f>Scenarios!$F$12</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>D&amp;A % of revenue</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="n"/>
-      <c r="F15" s="20">
-        <f>Scenarios!$F$12</f>
-        <v/>
-      </c>
-      <c r="G15" s="20">
-        <f>Scenarios!$F$12</f>
-        <v/>
-      </c>
-      <c r="H15" s="20">
-        <f>Scenarios!$F$12</f>
-        <v/>
-      </c>
-      <c r="I15" s="20">
-        <f>Scenarios!$F$12</f>
-        <v/>
-      </c>
-      <c r="J15" s="20">
-        <f>Scenarios!$F$12</f>
+          <t>Plus: depreciation &amp; amortization</t>
+        </is>
+      </c>
+      <c r="F15" s="75">
+        <f>Scenarios!F55</f>
+        <v/>
+      </c>
+      <c r="G15" s="75">
+        <f>Scenarios!F56</f>
+        <v/>
+      </c>
+      <c r="H15" s="75">
+        <f>Scenarios!F57</f>
+        <v/>
+      </c>
+      <c r="I15" s="75">
+        <f>Scenarios!F58</f>
+        <v/>
+      </c>
+      <c r="J15" s="75">
+        <f>Scenarios!F59</f>
+        <v/>
+      </c>
+      <c r="K15" s="86">
+        <f>IF(MAX(ABS(F16-Scenarios!$F$55),ABS(G16-Scenarios!$F$56),ABS(H16-Scenarios!$F$57),ABS(I16-Scenarios!$F$58),ABS(J16-Scenarios!$F$59))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Plus: depreciation &amp; amortization</t>
-        </is>
-      </c>
-      <c r="F16" s="75">
-        <f>Scenarios!F55</f>
-        <v/>
-      </c>
-      <c r="G16" s="75">
-        <f>Scenarios!F56</f>
-        <v/>
-      </c>
-      <c r="H16" s="75">
-        <f>Scenarios!F57</f>
-        <v/>
-      </c>
-      <c r="I16" s="75">
-        <f>Scenarios!F58</f>
-        <v/>
-      </c>
-      <c r="J16" s="75">
-        <f>Scenarios!F59</f>
-        <v/>
-      </c>
-      <c r="K16" s="86">
-        <f>IF(MAX(ABS(F16-Scenarios!$F$55),ABS(G16-Scenarios!$F$56),ABS(H16-Scenarios!$F$57),ABS(I16-Scenarios!$F$58),ABS(J16-Scenarios!$F$59))&lt;0.5,"OK","CHECK")</f>
+          <t>Capex % of revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="n"/>
+      <c r="F16" s="20">
+        <f>Scenarios!$F$13</f>
+        <v/>
+      </c>
+      <c r="G16" s="20">
+        <f>Scenarios!$F$13</f>
+        <v/>
+      </c>
+      <c r="H16" s="20">
+        <f>Scenarios!$F$13</f>
+        <v/>
+      </c>
+      <c r="I16" s="20">
+        <f>Scenarios!$F$13</f>
+        <v/>
+      </c>
+      <c r="J16" s="20">
+        <f>Scenarios!$F$13</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>Capex % of revenue</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="38" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="n"/>
-      <c r="F17" s="20">
-        <f>Scenarios!$F$13</f>
-        <v/>
-      </c>
-      <c r="G17" s="20">
-        <f>Scenarios!$F$13</f>
-        <v/>
-      </c>
-      <c r="H17" s="20">
-        <f>Scenarios!$F$13</f>
-        <v/>
-      </c>
-      <c r="I17" s="20">
-        <f>Scenarios!$F$13</f>
-        <v/>
-      </c>
-      <c r="J17" s="20">
-        <f>Scenarios!$F$13</f>
+          <t>Less: capital expenditures</t>
+        </is>
+      </c>
+      <c r="F17" s="75">
+        <f>-Scenarios!F60</f>
+        <v/>
+      </c>
+      <c r="G17" s="75">
+        <f>-Scenarios!F61</f>
+        <v/>
+      </c>
+      <c r="H17" s="75">
+        <f>-Scenarios!F62</f>
+        <v/>
+      </c>
+      <c r="I17" s="75">
+        <f>-Scenarios!F63</f>
+        <v/>
+      </c>
+      <c r="J17" s="75">
+        <f>-Scenarios!F64</f>
+        <v/>
+      </c>
+      <c r="K17" s="86">
+        <f>IF(MAX(ABS(F18+Scenarios!$F$60),ABS(G18+Scenarios!$F$61),ABS(H18+Scenarios!$F$62),ABS(I18+Scenarios!$F$63),ABS(J18+Scenarios!$F$64))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Less: capital expenditures</t>
-        </is>
-      </c>
-      <c r="F18" s="75">
-        <f>-Scenarios!F60</f>
-        <v/>
-      </c>
-      <c r="G18" s="75">
-        <f>-Scenarios!F61</f>
-        <v/>
-      </c>
-      <c r="H18" s="75">
-        <f>-Scenarios!F62</f>
-        <v/>
-      </c>
-      <c r="I18" s="75">
-        <f>-Scenarios!F63</f>
-        <v/>
-      </c>
-      <c r="J18" s="75">
-        <f>-Scenarios!F64</f>
+          <t>DSO (days) — flat vs FY25</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="88" t="n">
+        <v>6.267883648875038</v>
+      </c>
+      <c r="F18" s="28">
+        <f>Scenarios!F65</f>
+        <v/>
+      </c>
+      <c r="G18" s="28">
+        <f>Scenarios!F66</f>
+        <v/>
+      </c>
+      <c r="H18" s="28">
+        <f>Scenarios!F67</f>
+        <v/>
+      </c>
+      <c r="I18" s="28">
+        <f>Scenarios!F68</f>
+        <v/>
+      </c>
+      <c r="J18" s="28">
+        <f>Scenarios!F69</f>
         <v/>
       </c>
       <c r="K18" s="86">
-        <f>IF(MAX(ABS(F18+Scenarios!$F$60),ABS(G18+Scenarios!$F$61),ABS(H18+Scenarios!$F$62),ABS(I18+Scenarios!$F$63),ABS(J18+Scenarios!$F$64))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F20-Scenarios!$F$65),ABS(G20-Scenarios!$F$66),ABS(H20-Scenarios!$F$67),ABS(I20-Scenarios!$F$68),ABS(J20-Scenarios!$F$69))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="52" t="inlineStr">
-        <is>
-          <t>Working capital schedule (driver-based)  [click − to collapse detail]</t>
-        </is>
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="74" t="n">
+        <v>190657</v>
+      </c>
+      <c r="F19" s="75">
+        <f>Scenarios!F70</f>
+        <v/>
+      </c>
+      <c r="G19" s="75">
+        <f>Scenarios!F71</f>
+        <v/>
+      </c>
+      <c r="H19" s="75">
+        <f>Scenarios!F72</f>
+        <v/>
+      </c>
+      <c r="I19" s="75">
+        <f>Scenarios!F73</f>
+        <v/>
+      </c>
+      <c r="J19" s="75">
+        <f>Scenarios!F74</f>
+        <v/>
+      </c>
+      <c r="K19" s="86">
+        <f>IF(MAX(ABS(F21-Scenarios!$F$70),ABS(G21-Scenarios!$F$71),ABS(H21-Scenarios!$F$72),ABS(I21-Scenarios!$F$73),ABS(J21-Scenarios!$F$74))&lt;0.5,"OK","CHECK")</f>
+        <v/>
       </c>
     </row>
     <row r="20" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>DSO (days) — flat vs FY25</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="18" t="inlineStr">
+          <t>DIO (days) — FY25 anchor, −1 day/yr</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="38" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
       <c r="D20" s="19" t="n"/>
       <c r="E20" s="88" t="n">
-        <v>6.267883648875038</v>
+        <v>128.8324100108167</v>
       </c>
       <c r="F20" s="28">
-        <f>Scenarios!F65</f>
+        <f>Scenarios!F75</f>
         <v/>
       </c>
       <c r="G20" s="28">
-        <f>Scenarios!F66</f>
+        <f>Scenarios!F76</f>
         <v/>
       </c>
       <c r="H20" s="28">
-        <f>Scenarios!F67</f>
+        <f>Scenarios!F77</f>
         <v/>
       </c>
       <c r="I20" s="28">
-        <f>Scenarios!F68</f>
+        <f>Scenarios!F78</f>
         <v/>
       </c>
       <c r="J20" s="28">
-        <f>Scenarios!F69</f>
+        <f>Scenarios!F79</f>
         <v/>
       </c>
       <c r="K20" s="86">
-        <f>IF(MAX(ABS(F20-Scenarios!$F$65),ABS(G20-Scenarios!$F$66),ABS(H20-Scenarios!$F$67),ABS(I20-Scenarios!$F$68),ABS(J20-Scenarios!$F$69))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F22-Scenarios!$F$75),ABS(G22-Scenarios!$F$76),ABS(H22-Scenarios!$F$77),ABS(I22-Scenarios!$F$78),ABS(J22-Scenarios!$F$79))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Accounts receivable, net</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B21" s="17" t="n"/>
@@ -9201,78 +9250,78 @@
       </c>
       <c r="D21" s="19" t="n"/>
       <c r="E21" s="74" t="n">
-        <v>190657</v>
+        <v>1700753</v>
       </c>
       <c r="F21" s="75">
-        <f>Scenarios!F70</f>
+        <f>Scenarios!F80</f>
         <v/>
       </c>
       <c r="G21" s="75">
-        <f>Scenarios!F71</f>
+        <f>Scenarios!F81</f>
         <v/>
       </c>
       <c r="H21" s="75">
-        <f>Scenarios!F72</f>
+        <f>Scenarios!F82</f>
         <v/>
       </c>
       <c r="I21" s="75">
-        <f>Scenarios!F73</f>
+        <f>Scenarios!F83</f>
         <v/>
       </c>
       <c r="J21" s="75">
-        <f>Scenarios!F74</f>
+        <f>Scenarios!F84</f>
         <v/>
       </c>
       <c r="K21" s="86">
-        <f>IF(MAX(ABS(F21-Scenarios!$F$70),ABS(G21-Scenarios!$F$71),ABS(H21-Scenarios!$F$72),ABS(I21-Scenarios!$F$73),ABS(J21-Scenarios!$F$74))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F23-Scenarios!$F$80),ABS(G23-Scenarios!$F$81),ABS(H23-Scenarios!$F$82),ABS(I23-Scenarios!$F$83),ABS(J23-Scenarios!$F$84))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="22" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>DIO (days) — FY25 anchor, −1 day/yr</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="38" t="inlineStr">
+          <t>DPO (days) — flat vs FY25</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
       <c r="D22" s="19" t="n"/>
       <c r="E22" s="88" t="n">
-        <v>128.8324100108167</v>
+        <v>25.10521290169407</v>
       </c>
       <c r="F22" s="28">
-        <f>Scenarios!F75</f>
+        <f>Scenarios!F85</f>
         <v/>
       </c>
       <c r="G22" s="28">
-        <f>Scenarios!F76</f>
+        <f>Scenarios!F86</f>
         <v/>
       </c>
       <c r="H22" s="28">
-        <f>Scenarios!F77</f>
+        <f>Scenarios!F87</f>
         <v/>
       </c>
       <c r="I22" s="28">
-        <f>Scenarios!F78</f>
+        <f>Scenarios!F88</f>
         <v/>
       </c>
       <c r="J22" s="28">
-        <f>Scenarios!F79</f>
+        <f>Scenarios!F89</f>
         <v/>
       </c>
       <c r="K22" s="86">
-        <f>IF(MAX(ABS(F22-Scenarios!$F$75),ABS(G22-Scenarios!$F$76),ABS(H22-Scenarios!$F$77),ABS(I22-Scenarios!$F$78),ABS(J22-Scenarios!$F$79))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F24-Scenarios!$F$85),ABS(G24-Scenarios!$F$86),ABS(H24-Scenarios!$F$87),ABS(I24-Scenarios!$F$88),ABS(J24-Scenarios!$F$89))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="23" hidden="1" outlineLevel="1" ht="112" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Accounts payable</t>
         </is>
       </c>
       <c r="B23" s="17" t="n"/>
@@ -9283,37 +9332,37 @@
       </c>
       <c r="D23" s="19" t="n"/>
       <c r="E23" s="74" t="n">
-        <v>1700753</v>
+        <v>331421</v>
       </c>
       <c r="F23" s="75">
-        <f>Scenarios!F80</f>
+        <f>Scenarios!F90</f>
         <v/>
       </c>
       <c r="G23" s="75">
-        <f>Scenarios!F81</f>
+        <f>Scenarios!F91</f>
         <v/>
       </c>
       <c r="H23" s="75">
-        <f>Scenarios!F82</f>
+        <f>Scenarios!F92</f>
         <v/>
       </c>
       <c r="I23" s="75">
-        <f>Scenarios!F83</f>
+        <f>Scenarios!F93</f>
         <v/>
       </c>
       <c r="J23" s="75">
-        <f>Scenarios!F84</f>
+        <f>Scenarios!F94</f>
         <v/>
       </c>
       <c r="K23" s="86">
-        <f>IF(MAX(ABS(F23-Scenarios!$F$80),ABS(G23-Scenarios!$F$81),ABS(H23-Scenarios!$F$82),ABS(I23-Scenarios!$F$83),ABS(J23-Scenarios!$F$84))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F25-Scenarios!$F$90),ABS(G25-Scenarios!$F$91),ABS(H25-Scenarios!$F$92),ABS(I25-Scenarios!$F$93),ABS(J25-Scenarios!$F$94))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="24" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>DPO (days) — flat vs FY25</t>
+          <t>Prepaid expenses (% of revenue)</t>
         </is>
       </c>
       <c r="B24" s="17" t="n"/>
@@ -9323,38 +9372,34 @@
         </is>
       </c>
       <c r="D24" s="19" t="n"/>
-      <c r="E24" s="88" t="n">
-        <v>25.10521290169407</v>
-      </c>
-      <c r="F24" s="28">
-        <f>Scenarios!F85</f>
-        <v/>
-      </c>
-      <c r="G24" s="28">
-        <f>Scenarios!F86</f>
-        <v/>
-      </c>
-      <c r="H24" s="28">
-        <f>Scenarios!F87</f>
-        <v/>
-      </c>
-      <c r="I24" s="28">
-        <f>Scenarios!F88</f>
-        <v/>
-      </c>
-      <c r="J24" s="28">
-        <f>Scenarios!F89</f>
-        <v/>
-      </c>
-      <c r="K24" s="86">
-        <f>IF(MAX(ABS(F24-Scenarios!$F$85),ABS(G24-Scenarios!$F$86),ABS(H24-Scenarios!$F$87),ABS(I24-Scenarios!$F$88),ABS(J24-Scenarios!$F$89))&lt;0.5,"OK","CHECK")</f>
+      <c r="E24" s="77" t="n">
+        <v>0.05080692810692991</v>
+      </c>
+      <c r="F24" s="20">
+        <f>Scenarios!$F$19</f>
+        <v/>
+      </c>
+      <c r="G24" s="20">
+        <f>Scenarios!$F$19</f>
+        <v/>
+      </c>
+      <c r="H24" s="20">
+        <f>Scenarios!$F$19</f>
+        <v/>
+      </c>
+      <c r="I24" s="20">
+        <f>Scenarios!$F$19</f>
+        <v/>
+      </c>
+      <c r="J24" s="20">
+        <f>Scenarios!$F$19</f>
         <v/>
       </c>
     </row>
     <row r="25" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Accounts payable</t>
+          <t>Prepaid expenses (other current assets)</t>
         </is>
       </c>
       <c r="B25" s="17" t="n"/>
@@ -9365,37 +9410,37 @@
       </c>
       <c r="D25" s="19" t="n"/>
       <c r="E25" s="74" t="n">
-        <v>331421</v>
+        <v>564089</v>
       </c>
       <c r="F25" s="75">
-        <f>Scenarios!F90</f>
+        <f>Scenarios!F95</f>
         <v/>
       </c>
       <c r="G25" s="75">
-        <f>Scenarios!F91</f>
+        <f>Scenarios!F96</f>
         <v/>
       </c>
       <c r="H25" s="75">
-        <f>Scenarios!F92</f>
+        <f>Scenarios!F97</f>
         <v/>
       </c>
       <c r="I25" s="75">
-        <f>Scenarios!F93</f>
+        <f>Scenarios!F98</f>
         <v/>
       </c>
       <c r="J25" s="75">
-        <f>Scenarios!F94</f>
+        <f>Scenarios!F99</f>
         <v/>
       </c>
       <c r="K25" s="86">
-        <f>IF(MAX(ABS(F25-Scenarios!$F$90),ABS(G25-Scenarios!$F$91),ABS(H25-Scenarios!$F$92),ABS(I25-Scenarios!$F$93),ABS(J25-Scenarios!$F$94))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F27-Scenarios!$F$95),ABS(G27-Scenarios!$F$96),ABS(H27-Scenarios!$F$97),ABS(I27-Scenarios!$F$98),ABS(J27-Scenarios!$F$99))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="26" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Prepaid expenses (% of revenue)</t>
+          <t>Accrued liabilities (% of revenue)</t>
         </is>
       </c>
       <c r="B26" s="17" t="n"/>
@@ -9406,33 +9451,33 @@
       </c>
       <c r="D26" s="19" t="n"/>
       <c r="E26" s="77" t="n">
-        <v>0.05080692810692991</v>
+        <v>0.05971412101669879</v>
       </c>
       <c r="F26" s="20">
-        <f>Scenarios!$F$19</f>
+        <f>Scenarios!$F$20</f>
         <v/>
       </c>
       <c r="G26" s="20">
-        <f>Scenarios!$F$19</f>
+        <f>Scenarios!$F$20</f>
         <v/>
       </c>
       <c r="H26" s="20">
-        <f>Scenarios!$F$19</f>
+        <f>Scenarios!$F$20</f>
         <v/>
       </c>
       <c r="I26" s="20">
-        <f>Scenarios!$F$19</f>
+        <f>Scenarios!$F$20</f>
         <v/>
       </c>
       <c r="J26" s="20">
-        <f>Scenarios!$F$19</f>
+        <f>Scenarios!$F$20</f>
         <v/>
       </c>
     </row>
     <row r="27" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets)</t>
+          <t>Accrued liabilities and other</t>
         </is>
       </c>
       <c r="B27" s="17" t="n"/>
@@ -9443,153 +9488,154 @@
       </c>
       <c r="D27" s="19" t="n"/>
       <c r="E27" s="74" t="n">
-        <v>564089</v>
+        <v>662982</v>
       </c>
       <c r="F27" s="75">
-        <f>Scenarios!F95</f>
+        <f>Scenarios!F100</f>
         <v/>
       </c>
       <c r="G27" s="75">
-        <f>Scenarios!F96</f>
+        <f>Scenarios!F101</f>
         <v/>
       </c>
       <c r="H27" s="75">
-        <f>Scenarios!F97</f>
+        <f>Scenarios!F102</f>
         <v/>
       </c>
       <c r="I27" s="75">
-        <f>Scenarios!F98</f>
+        <f>Scenarios!F103</f>
         <v/>
       </c>
       <c r="J27" s="75">
-        <f>Scenarios!F99</f>
+        <f>Scenarios!F104</f>
         <v/>
       </c>
       <c r="K27" s="86">
-        <f>IF(MAX(ABS(F27-Scenarios!$F$95),ABS(G27-Scenarios!$F$96),ABS(H27-Scenarios!$F$97),ABS(I27-Scenarios!$F$98),ABS(J27-Scenarios!$F$99))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F29-Scenarios!$F$100),ABS(G29-Scenarios!$F$101),ABS(H29-Scenarios!$F$102),ABS(I29-Scenarios!$F$103),ABS(J29-Scenarios!$F$104))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="28" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Accrued liabilities (% of revenue)</t>
+          <t>Current operating assets (AR + inv + prepaids)</t>
         </is>
       </c>
       <c r="B28" s="17" t="n"/>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>Scenarios</t>
         </is>
       </c>
       <c r="D28" s="19" t="n"/>
-      <c r="E28" s="77" t="n">
-        <v>0.05971412101669879</v>
-      </c>
-      <c r="F28" s="20">
-        <f>Scenarios!$F$20</f>
-        <v/>
-      </c>
-      <c r="G28" s="20">
-        <f>Scenarios!$F$20</f>
-        <v/>
-      </c>
-      <c r="H28" s="20">
-        <f>Scenarios!$F$20</f>
-        <v/>
-      </c>
-      <c r="I28" s="20">
-        <f>Scenarios!$F$20</f>
-        <v/>
-      </c>
-      <c r="J28" s="20">
-        <f>Scenarios!$F$20</f>
+      <c r="F28" s="75">
+        <f>Scenarios!F105</f>
+        <v/>
+      </c>
+      <c r="G28" s="75">
+        <f>Scenarios!F106</f>
+        <v/>
+      </c>
+      <c r="H28" s="75">
+        <f>Scenarios!F107</f>
+        <v/>
+      </c>
+      <c r="I28" s="75">
+        <f>Scenarios!F108</f>
+        <v/>
+      </c>
+      <c r="J28" s="75">
+        <f>Scenarios!F109</f>
+        <v/>
+      </c>
+      <c r="K28" s="86">
+        <f>IF(MAX(ABS(F30-Scenarios!$F$105),ABS(G30-Scenarios!$F$106),ABS(H30-Scenarios!$F$107),ABS(I30-Scenarios!$F$108),ABS(J30-Scenarios!$F$109))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="29" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Accrued liabilities and other</t>
+          <t>Current operating liabilities (AP + accruals)</t>
         </is>
       </c>
       <c r="B29" s="17" t="n"/>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>Scenarios</t>
         </is>
       </c>
       <c r="D29" s="19" t="n"/>
-      <c r="E29" s="74" t="n">
-        <v>662982</v>
-      </c>
       <c r="F29" s="75">
-        <f>Scenarios!F100</f>
+        <f>Scenarios!F110</f>
         <v/>
       </c>
       <c r="G29" s="75">
-        <f>Scenarios!F101</f>
+        <f>Scenarios!F111</f>
         <v/>
       </c>
       <c r="H29" s="75">
-        <f>Scenarios!F102</f>
+        <f>Scenarios!F112</f>
         <v/>
       </c>
       <c r="I29" s="75">
-        <f>Scenarios!F103</f>
+        <f>Scenarios!F113</f>
         <v/>
       </c>
       <c r="J29" s="75">
-        <f>Scenarios!F104</f>
+        <f>Scenarios!F114</f>
         <v/>
       </c>
       <c r="K29" s="86">
-        <f>IF(MAX(ABS(F29-Scenarios!$F$100),ABS(G29-Scenarios!$F$101),ABS(H29-Scenarios!$F$102),ABS(I29-Scenarios!$F$103),ABS(J29-Scenarios!$F$104))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F31-Scenarios!$F$110),ABS(G31-Scenarios!$F$111),ABS(H31-Scenarios!$F$112),ABS(I31-Scenarios!$F$113),ABS(J31-Scenarios!$F$114))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="30" hidden="1" outlineLevel="1" ht="42" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Current operating assets (AR + inv + prepaids)</t>
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>Net working capital</t>
         </is>
       </c>
       <c r="B30" s="17" t="n"/>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>Scenarios</t>
+          <t>10-K</t>
         </is>
       </c>
       <c r="D30" s="19" t="n"/>
-      <c r="F30" s="75">
-        <f>Scenarios!F105</f>
-        <v/>
-      </c>
-      <c r="G30" s="75">
-        <f>Scenarios!F106</f>
-        <v/>
-      </c>
-      <c r="H30" s="75">
-        <f>Scenarios!F107</f>
-        <v/>
-      </c>
-      <c r="I30" s="75">
-        <f>Scenarios!F108</f>
-        <v/>
-      </c>
-      <c r="J30" s="75">
-        <f>Scenarios!F109</f>
-        <v/>
-      </c>
-      <c r="K30" s="86">
-        <f>IF(MAX(ABS(F30-Scenarios!$F$105),ABS(G30-Scenarios!$F$106),ABS(H30-Scenarios!$F$107),ABS(I30-Scenarios!$F$108),ABS(J30-Scenarios!$F$109))&lt;0.5,"OK","CHECK")</f>
+      <c r="E30" s="76" t="n">
+        <v>1461096</v>
+      </c>
+      <c r="F30" s="25">
+        <f>Scenarios!F115</f>
+        <v/>
+      </c>
+      <c r="G30" s="25">
+        <f>Scenarios!F116</f>
+        <v/>
+      </c>
+      <c r="H30" s="25">
+        <f>Scenarios!F117</f>
+        <v/>
+      </c>
+      <c r="I30" s="25">
+        <f>Scenarios!F118</f>
+        <v/>
+      </c>
+      <c r="J30" s="25">
+        <f>Scenarios!F119</f>
+        <v/>
+      </c>
+      <c r="K30" s="87">
+        <f>IF(MAX(ABS(F32-Scenarios!$F$115),ABS(G32-Scenarios!$F$116),ABS(H32-Scenarios!$F$117),ABS(I32-Scenarios!$F$118),ABS(J32-Scenarios!$F$119))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="31" hidden="1" outlineLevel="1" ht="42" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Current operating liabilities (AP + accruals)</t>
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>ΔNWC (prior yr − current yr)</t>
         </is>
       </c>
       <c r="B31" s="17" t="n"/>
@@ -9599,1013 +9645,1020 @@
         </is>
       </c>
       <c r="D31" s="19" t="n"/>
-      <c r="F31" s="75">
-        <f>Scenarios!F110</f>
-        <v/>
-      </c>
-      <c r="G31" s="75">
-        <f>Scenarios!F111</f>
-        <v/>
-      </c>
-      <c r="H31" s="75">
-        <f>Scenarios!F112</f>
-        <v/>
-      </c>
-      <c r="I31" s="75">
-        <f>Scenarios!F113</f>
-        <v/>
-      </c>
-      <c r="J31" s="75">
-        <f>Scenarios!F114</f>
-        <v/>
-      </c>
-      <c r="K31" s="86">
-        <f>IF(MAX(ABS(F31-Scenarios!$F$110),ABS(G31-Scenarios!$F$111),ABS(H31-Scenarios!$F$112),ABS(I31-Scenarios!$F$113),ABS(J31-Scenarios!$F$114))&lt;0.5,"OK","CHECK")</f>
+      <c r="F31" s="25">
+        <f>Scenarios!F120</f>
+        <v/>
+      </c>
+      <c r="G31" s="25">
+        <f>Scenarios!F121</f>
+        <v/>
+      </c>
+      <c r="H31" s="25">
+        <f>Scenarios!F122</f>
+        <v/>
+      </c>
+      <c r="I31" s="25">
+        <f>Scenarios!F123</f>
+        <v/>
+      </c>
+      <c r="J31" s="25">
+        <f>Scenarios!F124</f>
+        <v/>
+      </c>
+      <c r="K31" s="87">
+        <f>IF(MAX(ABS(F33-Scenarios!$F$120),ABS(G33-Scenarios!$F$121),ABS(H33-Scenarios!$F$122),ABS(I33-Scenarios!$F$123),ABS(J33-Scenarios!$F$124))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="32" hidden="1" outlineLevel="1" ht="42" customHeight="1">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>Net working capital</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="76" t="n">
-        <v>1461096</v>
-      </c>
-      <c r="F32" s="25">
-        <f>Scenarios!F115</f>
-        <v/>
-      </c>
-      <c r="G32" s="25">
-        <f>Scenarios!F116</f>
-        <v/>
-      </c>
-      <c r="H32" s="25">
-        <f>Scenarios!F117</f>
-        <v/>
-      </c>
-      <c r="I32" s="25">
-        <f>Scenarios!F118</f>
-        <v/>
-      </c>
-      <c r="J32" s="25">
-        <f>Scenarios!F119</f>
+          <t>Unlevered free cash flow</t>
+        </is>
+      </c>
+      <c r="F32" s="89">
+        <f>Scenarios!F125</f>
+        <v/>
+      </c>
+      <c r="G32" s="89">
+        <f>Scenarios!F126</f>
+        <v/>
+      </c>
+      <c r="H32" s="89">
+        <f>Scenarios!F127</f>
+        <v/>
+      </c>
+      <c r="I32" s="89">
+        <f>Scenarios!F128</f>
+        <v/>
+      </c>
+      <c r="J32" s="89">
+        <f>Scenarios!F129</f>
         <v/>
       </c>
       <c r="K32" s="87">
-        <f>IF(MAX(ABS(F32-Scenarios!$F$115),ABS(G32-Scenarios!$F$116),ABS(H32-Scenarios!$F$117),ABS(I32-Scenarios!$F$118),ABS(J32-Scenarios!$F$119))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F35-Scenarios!$F$125),ABS(G35-Scenarios!$F$126),ABS(H35-Scenarios!$F$127),ABS(I35-Scenarios!$F$128),ABS(J35-Scenarios!$F$129))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="56" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
-        <is>
-          <t>ΔNWC (prior yr − current yr)</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>Scenarios</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="n"/>
-      <c r="F33" s="25">
-        <f>Scenarios!F120</f>
-        <v/>
-      </c>
-      <c r="G33" s="25">
-        <f>Scenarios!F121</f>
-        <v/>
-      </c>
-      <c r="H33" s="25">
-        <f>Scenarios!F122</f>
-        <v/>
-      </c>
-      <c r="I33" s="25">
-        <f>Scenarios!F123</f>
-        <v/>
-      </c>
-      <c r="J33" s="25">
-        <f>Scenarios!F124</f>
-        <v/>
-      </c>
-      <c r="K33" s="87">
-        <f>IF(MAX(ABS(F33-Scenarios!$F$120),ABS(G33-Scenarios!$F$121),ABS(H33-Scenarios!$F$122),ABS(I33-Scenarios!$F$123),ABS(J33-Scenarios!$F$124))&lt;0.5,"OK","CHECK")</f>
-        <v/>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Discount period (years)</t>
+        </is>
+      </c>
+      <c r="F33" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="90" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
-        <is>
-          <t>Unlevered free cash flow</t>
-        </is>
-      </c>
-      <c r="F34" s="89">
-        <f>Scenarios!F125</f>
-        <v/>
-      </c>
-      <c r="G34" s="89">
-        <f>Scenarios!F126</f>
-        <v/>
-      </c>
-      <c r="H34" s="89">
-        <f>Scenarios!F127</f>
-        <v/>
-      </c>
-      <c r="I34" s="89">
-        <f>Scenarios!F128</f>
-        <v/>
-      </c>
-      <c r="J34" s="89">
-        <f>Scenarios!F129</f>
-        <v/>
-      </c>
-      <c r="K34" s="87">
-        <f>IF(MAX(ABS(F35-Scenarios!$F$125),ABS(G35-Scenarios!$F$126),ABS(H35-Scenarios!$F$127),ABS(I35-Scenarios!$F$128),ABS(J35-Scenarios!$F$129))&lt;0.5,"OK","CHECK")</f>
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Discount factor @ WACC</t>
+        </is>
+      </c>
+      <c r="F34" s="91">
+        <f>1/(1+Scenarios!$F$9)^F36</f>
+        <v/>
+      </c>
+      <c r="G34" s="91">
+        <f>1/(1+Scenarios!$F$9)^G36</f>
+        <v/>
+      </c>
+      <c r="H34" s="91">
+        <f>1/(1+Scenarios!$F$9)^H36</f>
+        <v/>
+      </c>
+      <c r="I34" s="91">
+        <f>1/(1+Scenarios!$F$9)^I36</f>
+        <v/>
+      </c>
+      <c r="J34" s="91">
+        <f>1/(1+Scenarios!$F$9)^J36</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Discount period (years)</t>
-        </is>
-      </c>
-      <c r="F35" s="90" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="90" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" s="90" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" s="90" t="n">
-        <v>4</v>
-      </c>
-      <c r="J35" s="90" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Discount factor @ WACC</t>
-        </is>
-      </c>
-      <c r="F36" s="91">
-        <f>1/(1+Scenarios!$F$9)^F36</f>
-        <v/>
-      </c>
-      <c r="G36" s="91">
-        <f>1/(1+Scenarios!$F$9)^G36</f>
-        <v/>
-      </c>
-      <c r="H36" s="91">
-        <f>1/(1+Scenarios!$F$9)^H36</f>
-        <v/>
-      </c>
-      <c r="I36" s="91">
-        <f>1/(1+Scenarios!$F$9)^I36</f>
-        <v/>
-      </c>
-      <c r="J36" s="91">
-        <f>1/(1+Scenarios!$F$9)^J36</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>PV of unlevered FCF</t>
+        </is>
+      </c>
+      <c r="F35" s="25">
+        <f>F35*F37</f>
+        <v/>
+      </c>
+      <c r="G35" s="25">
+        <f>G35*G37</f>
+        <v/>
+      </c>
+      <c r="H35" s="25">
+        <f>H35*H37</f>
+        <v/>
+      </c>
+      <c r="I35" s="25">
+        <f>I35*I37</f>
+        <v/>
+      </c>
+      <c r="J35" s="25">
+        <f>J35*J37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
-        <is>
-          <t>PV of unlevered FCF</t>
-        </is>
-      </c>
-      <c r="F37" s="25">
-        <f>F35*F37</f>
-        <v/>
-      </c>
-      <c r="G37" s="25">
-        <f>G35*G37</f>
-        <v/>
-      </c>
-      <c r="H37" s="25">
-        <f>H35*H37</f>
-        <v/>
-      </c>
-      <c r="I37" s="25">
-        <f>I35*I37</f>
-        <v/>
-      </c>
-      <c r="J37" s="25">
-        <f>J35*J37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38"/>
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>Scenarios linkage summary (column K should all read OK)</t>
+        </is>
+      </c>
+      <c r="K37" s="92">
+        <f>IF(COUNTIF(K5:K35,"CHECK")=0,"ALL OK","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="93" t="inlineStr">
+        <is>
+          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="13" t="n"/>
+    </row>
     <row r="39">
-      <c r="A39" s="15" t="inlineStr">
-        <is>
-          <t>Scenarios linkage summary (column K should all read OK)</t>
-        </is>
-      </c>
-      <c r="K39" s="92">
-        <f>IF(COUNTIF(K5:K35,"CHECK")=0,"ALL OK","REVIEW")</f>
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>Sum of PV of explicit FCF (FY26–FY30)</t>
+        </is>
+      </c>
+      <c r="E39" s="70">
+        <f>SUM(F38:J38)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="93" t="inlineStr">
-        <is>
-          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="n"/>
-      <c r="C40" s="13" t="n"/>
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Terminal growth rate (g)</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>FRED</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="32">
+        <f>Scenarios!$F$10</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>Sum of PV of explicit FCF (FY26–FY30)</t>
-        </is>
-      </c>
-      <c r="E41" s="70">
-        <f>SUM(F38:J38)</f>
+          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
+        </is>
+      </c>
+      <c r="E41" s="25">
+        <f>J11+J16</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
         <is>
-          <t>Terminal growth rate (g)</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="n"/>
-      <c r="C42" s="18" t="inlineStr">
-        <is>
-          <t>FRED</t>
-        </is>
-      </c>
-      <c r="D42" s="19" t="n"/>
-      <c r="E42" s="32">
-        <f>Scenarios!$F$10</f>
+          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+        </is>
+      </c>
+      <c r="E42" s="75">
+        <f>J35*(1+Scenarios!$F$10)/(Scenarios!$F$9-Scenarios!$F$10)</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="23" t="inlineStr">
-        <is>
-          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
-        </is>
-      </c>
-      <c r="E43" s="25">
-        <f>J11+J16</f>
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
+        </is>
+      </c>
+      <c r="E43" s="94">
+        <f>E42/E41</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
-        </is>
-      </c>
-      <c r="E44" s="75">
-        <f>J35*(1+Scenarios!$F$10)/(Scenarios!$F$9-Scenarios!$F$10)</f>
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E44" s="70">
+        <f>E42/(1+Scenarios!$F$9)^J36</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
-        </is>
-      </c>
-      <c r="E45" s="94">
-        <f>E44/E43</f>
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise value</t>
+        </is>
+      </c>
+      <c r="E45" s="25">
+        <f>E39+E44</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E46" s="70">
-        <f>E44/(1+Scenarios!$F$9)^J36</f>
-        <v/>
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Plus: cash &amp; equivalents (FY2025)</t>
+        </is>
+      </c>
+      <c r="C46" s="95" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="74" t="n">
+        <v>1807202</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="inlineStr">
-        <is>
-          <t>Enterprise value</t>
-        </is>
-      </c>
-      <c r="E47" s="25">
-        <f>E41+E46</f>
-        <v/>
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>Less: total debt &amp; operating leases</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="n"/>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="n"/>
+      <c r="E47" s="74" t="n">
+        <v>-1798441</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>Plus: cash &amp; equivalents (FY2025)</t>
-        </is>
-      </c>
-      <c r="C48" s="95" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D48" s="19" t="n"/>
-      <c r="E48" s="74" t="n">
-        <v>1807202</v>
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>Equity value</t>
+        </is>
+      </c>
+      <c r="E48" s="25">
+        <f>E45+E46+E47</f>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Less: total debt &amp; operating leases</t>
-        </is>
-      </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="18" t="inlineStr">
+          <t>Shares outstanding (000)</t>
+        </is>
+      </c>
+      <c r="C49" s="95" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
       <c r="D49" s="19" t="n"/>
       <c r="E49" s="74" t="n">
-        <v>-1798441</v>
+        <v>111380</v>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="23" t="inlineStr">
         <is>
-          <t>Equity value</t>
-        </is>
-      </c>
-      <c r="E50" s="25">
-        <f>E47+E48+E49</f>
+          <t>Implied value per share</t>
+        </is>
+      </c>
+      <c r="E50" s="96">
+        <f>E48/E49</f>
+        <v/>
+      </c>
+      <c r="K50" s="87">
+        <f>IF(ABS(E56-Scenarios!$F$132)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>Shares outstanding (000)</t>
+          <t>Current share price</t>
         </is>
       </c>
       <c r="C51" s="95" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D51" s="19" t="n"/>
-      <c r="E51" s="74" t="n">
-        <v>111380</v>
+      <c r="E51" s="97" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="23" t="inlineStr">
         <is>
-          <t>Implied value per share</t>
-        </is>
-      </c>
-      <c r="E52" s="96">
-        <f>E50/E51</f>
-        <v/>
-      </c>
-      <c r="K52" s="87">
-        <f>IF(ABS(E56-Scenarios!$F$132)&lt;0.05,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>Current share price</t>
-        </is>
-      </c>
-      <c r="C53" s="95" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
-      <c r="D53" s="19" t="n"/>
-      <c r="E53" s="97" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="23" t="inlineStr">
-        <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E54" s="98">
-        <f>E52/E53-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="28" customHeight="1"/>
+      <c r="E52" s="98">
+        <f>E50/E51-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="93" t="inlineStr">
+        <is>
+          <t>SHARE REPURCHASE &amp; EPS ACCRETION SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="13" t="n"/>
+      <c r="D55" s="13" t="n"/>
+      <c r="E55" s="13" t="n"/>
+    </row>
     <row r="56"/>
     <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="93" t="inlineStr">
-        <is>
-          <t>SHARE REPURCHASE &amp; EPS ACCRETION SCHEDULE</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="n"/>
-      <c r="C57" s="13" t="n"/>
-      <c r="D57" s="13" t="n"/>
-      <c r="E57" s="13" t="n"/>
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>Annual repurchase budget ($000) — base case</t>
+        </is>
+      </c>
+      <c r="E57" s="37" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F57" s="37">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="G57" s="37">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="H57" s="37">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="I57" s="37">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="J57" s="37">
+        <f>$E$65</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="26" t="inlineStr">
-        <is>
-          <t>Guardrail: implied value per share above still divides equity value by Day-1 shares (E51 = 111,380k). This schedule does not change intrinsic DCF per share.</t>
-        </is>
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>Cost of equity — share-price growth rate</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="F58" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="G58" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="H58" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="I58" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="J58" s="20">
+        <f>$E$66</f>
+        <v/>
       </c>
     </row>
     <row r="59"/>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>Annual repurchase budget ($000) — base case</t>
-        </is>
-      </c>
-      <c r="E60" s="37" t="n">
-        <v>500000</v>
-      </c>
-      <c r="F60" s="37">
-        <f>$E$65</f>
-        <v/>
-      </c>
-      <c r="G60" s="37">
-        <f>$E$65</f>
-        <v/>
-      </c>
-      <c r="H60" s="37">
-        <f>$E$65</f>
-        <v/>
-      </c>
-      <c r="I60" s="37">
-        <f>$E$65</f>
-        <v/>
-      </c>
-      <c r="J60" s="37">
-        <f>$E$65</f>
+          <t>Unlevered free cash flow (from DCF above)</t>
+        </is>
+      </c>
+      <c r="F60" s="75">
+        <f>F35</f>
+        <v/>
+      </c>
+      <c r="G60" s="75">
+        <f>G35</f>
+        <v/>
+      </c>
+      <c r="H60" s="75">
+        <f>H35</f>
+        <v/>
+      </c>
+      <c r="I60" s="75">
+        <f>I35</f>
+        <v/>
+      </c>
+      <c r="J60" s="75">
+        <f>J35</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Cost of equity — share-price growth rate</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="F61" s="20">
-        <f>$E$66</f>
-        <v/>
-      </c>
-      <c r="G61" s="20">
-        <f>$E$66</f>
-        <v/>
-      </c>
-      <c r="H61" s="20">
-        <f>$E$66</f>
-        <v/>
-      </c>
-      <c r="I61" s="20">
-        <f>$E$66</f>
-        <v/>
-      </c>
-      <c r="J61" s="20">
-        <f>$E$66</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62"/>
-    <row r="63">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>Unlevered free cash flow (from DCF above)</t>
-        </is>
-      </c>
-      <c r="F63" s="75">
-        <f>F35</f>
-        <v/>
-      </c>
-      <c r="G63" s="75">
-        <f>G35</f>
-        <v/>
-      </c>
-      <c r="H63" s="75">
-        <f>H35</f>
-        <v/>
-      </c>
-      <c r="I63" s="75">
-        <f>I35</f>
-        <v/>
-      </c>
-      <c r="J63" s="75">
-        <f>J35</f>
-        <v/>
-      </c>
-    </row>
+          <t>Repurchase cash deployed (= fixed budget)</t>
+        </is>
+      </c>
+      <c r="E61" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="75">
+        <f>F65</f>
+        <v/>
+      </c>
+      <c r="G61" s="75">
+        <f>G65</f>
+        <v/>
+      </c>
+      <c r="H61" s="75">
+        <f>H65</f>
+        <v/>
+      </c>
+      <c r="I61" s="75">
+        <f>I65</f>
+        <v/>
+      </c>
+      <c r="J61" s="75">
+        <f>J65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t>Repurchase as % of UFCF (derived)</t>
+        </is>
+      </c>
+      <c r="F62" s="32">
+        <f>F69/F68</f>
+        <v/>
+      </c>
+      <c r="G62" s="32">
+        <f>G69/G68</f>
+        <v/>
+      </c>
+      <c r="H62" s="32">
+        <f>H69/H68</f>
+        <v/>
+      </c>
+      <c r="I62" s="32">
+        <f>I69/I68</f>
+        <v/>
+      </c>
+      <c r="J62" s="32">
+        <f>J69/J68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63"/>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>Repurchase cash deployed (= fixed budget)</t>
-        </is>
-      </c>
-      <c r="E64" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F64" s="75">
-        <f>F65</f>
-        <v/>
-      </c>
-      <c r="G64" s="75">
-        <f>G65</f>
-        <v/>
-      </c>
-      <c r="H64" s="75">
-        <f>H65</f>
-        <v/>
-      </c>
-      <c r="I64" s="75">
-        <f>I65</f>
-        <v/>
-      </c>
-      <c r="J64" s="75">
-        <f>J65</f>
+          <t>Projected share price ($)</t>
+        </is>
+      </c>
+      <c r="E64" s="99" t="n">
+        <v>100</v>
+      </c>
+      <c r="F64" s="99">
+        <f>E72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="G64" s="99">
+        <f>F72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="H64" s="99">
+        <f>G72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="I64" s="99">
+        <f>H72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="J64" s="99">
+        <f>I72*(1+$E$66)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>Repurchase as % of UFCF (derived)</t>
-        </is>
-      </c>
-      <c r="F65" s="32">
-        <f>F69/F68</f>
-        <v/>
-      </c>
-      <c r="G65" s="32">
-        <f>G69/G68</f>
-        <v/>
-      </c>
-      <c r="H65" s="32">
-        <f>H69/H68</f>
-        <v/>
-      </c>
-      <c r="I65" s="32">
-        <f>I69/I68</f>
-        <v/>
-      </c>
-      <c r="J65" s="32">
-        <f>J69/J68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66"/>
+          <t>Shares retired (000)</t>
+        </is>
+      </c>
+      <c r="E65" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="75">
+        <f>F69/F72</f>
+        <v/>
+      </c>
+      <c r="G65" s="75">
+        <f>G69/G72</f>
+        <v/>
+      </c>
+      <c r="H65" s="75">
+        <f>H69/H72</f>
+        <v/>
+      </c>
+      <c r="I65" s="75">
+        <f>I69/I72</f>
+        <v/>
+      </c>
+      <c r="J65" s="75">
+        <f>J69/J72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>Beginning shares (000)</t>
+        </is>
+      </c>
+      <c r="E66" s="22" t="n">
+        <v>111380</v>
+      </c>
+      <c r="F66" s="75">
+        <f>$E$74</f>
+        <v/>
+      </c>
+      <c r="G66" s="75">
+        <f>F75</f>
+        <v/>
+      </c>
+      <c r="H66" s="75">
+        <f>G75</f>
+        <v/>
+      </c>
+      <c r="I66" s="75">
+        <f>H75</f>
+        <v/>
+      </c>
+      <c r="J66" s="75">
+        <f>I75</f>
+        <v/>
+      </c>
+    </row>
     <row r="67">
-      <c r="A67" s="16" t="inlineStr">
-        <is>
-          <t>Projected share price ($)</t>
-        </is>
-      </c>
-      <c r="E67" s="99" t="n">
-        <v>100</v>
-      </c>
-      <c r="F67" s="99">
-        <f>E72*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="G67" s="99">
-        <f>F72*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="H67" s="99">
-        <f>G72*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="I67" s="99">
-        <f>H72*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="J67" s="99">
-        <f>I72*(1+$E$66)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="16" t="inlineStr">
-        <is>
-          <t>Shares retired (000)</t>
-        </is>
-      </c>
-      <c r="E68" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="75">
-        <f>F69/F72</f>
-        <v/>
-      </c>
-      <c r="G68" s="75">
-        <f>G69/G72</f>
-        <v/>
-      </c>
-      <c r="H68" s="75">
-        <f>H69/H72</f>
-        <v/>
-      </c>
-      <c r="I68" s="75">
-        <f>I69/I72</f>
-        <v/>
-      </c>
-      <c r="J68" s="75">
-        <f>J69/J72</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>Ending shares (000)</t>
+        </is>
+      </c>
+      <c r="E67" s="100" t="n">
+        <v>111380</v>
+      </c>
+      <c r="F67" s="25">
+        <f>F74-F73</f>
+        <v/>
+      </c>
+      <c r="G67" s="25">
+        <f>G74-G73</f>
+        <v/>
+      </c>
+      <c r="H67" s="25">
+        <f>H74-H73</f>
+        <v/>
+      </c>
+      <c r="I67" s="25">
+        <f>I74-I73</f>
+        <v/>
+      </c>
+      <c r="J67" s="25">
+        <f>J74-J73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>Beginning shares (000)</t>
+          <t>Projected net income ($000)</t>
         </is>
       </c>
       <c r="E69" s="22" t="n">
-        <v>111380</v>
+        <v>1579183</v>
       </c>
       <c r="F69" s="75">
-        <f>$E$74</f>
+        <f>('NOPAT Bridge'!E36-'NOPAT Bridge'!E23)*(1-'NOPAT Bridge'!E$39)</f>
         <v/>
       </c>
       <c r="G69" s="75">
-        <f>F75</f>
+        <f>('NOPAT Bridge'!F36-'NOPAT Bridge'!F23)*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
       <c r="H69" s="75">
-        <f>G75</f>
+        <f>('NOPAT Bridge'!G36-'NOPAT Bridge'!G23)*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
       <c r="I69" s="75">
-        <f>H75</f>
+        <f>('NOPAT Bridge'!H36-'NOPAT Bridge'!H23)*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
       <c r="J69" s="75">
-        <f>I75</f>
+        <f>('NOPAT Bridge'!I36-'NOPAT Bridge'!I23)*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="23" t="inlineStr">
         <is>
-          <t>Ending shares (000)</t>
-        </is>
-      </c>
-      <c r="E70" s="100" t="n">
-        <v>111380</v>
-      </c>
-      <c r="F70" s="25">
-        <f>F74-F73</f>
-        <v/>
-      </c>
-      <c r="G70" s="25">
-        <f>G74-G73</f>
-        <v/>
-      </c>
-      <c r="H70" s="25">
-        <f>H74-H73</f>
-        <v/>
-      </c>
-      <c r="I70" s="25">
-        <f>I74-I73</f>
-        <v/>
-      </c>
-      <c r="J70" s="25">
-        <f>J74-J73</f>
+          <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
+        </is>
+      </c>
+      <c r="E70" s="101" t="n">
+        <v>14.1783354282636</v>
+      </c>
+      <c r="F70" s="101">
+        <f>F77/F75</f>
+        <v/>
+      </c>
+      <c r="G70" s="101">
+        <f>G77/G75</f>
+        <v/>
+      </c>
+      <c r="H70" s="101">
+        <f>H77/H75</f>
+        <v/>
+      </c>
+      <c r="I70" s="101">
+        <f>I77/I75</f>
+        <v/>
+      </c>
+      <c r="J70" s="101">
+        <f>J77/J75</f>
         <v/>
       </c>
     </row>
     <row r="71"/>
     <row r="72">
-      <c r="A72" s="16" t="inlineStr">
-        <is>
-          <t>Projected net income ($000)</t>
-        </is>
-      </c>
-      <c r="E72" s="22" t="n">
-        <v>1579183</v>
-      </c>
-      <c r="F72" s="75">
-        <f>('NOPAT Bridge'!E36-'NOPAT Bridge'!E23)*(1-'NOPAT Bridge'!E$39)</f>
-        <v/>
-      </c>
-      <c r="G72" s="75">
-        <f>('NOPAT Bridge'!F36-'NOPAT Bridge'!F23)*(1-'NOPAT Bridge'!F$39)</f>
-        <v/>
-      </c>
-      <c r="H72" s="75">
-        <f>('NOPAT Bridge'!G36-'NOPAT Bridge'!G23)*(1-'NOPAT Bridge'!G$39)</f>
-        <v/>
-      </c>
-      <c r="I72" s="75">
-        <f>('NOPAT Bridge'!H36-'NOPAT Bridge'!H23)*(1-'NOPAT Bridge'!H$39)</f>
-        <v/>
-      </c>
-      <c r="J72" s="75">
-        <f>('NOPAT Bridge'!I36-'NOPAT Bridge'!I23)*(1-'NOPAT Bridge'!I$39)</f>
-        <v/>
-      </c>
+      <c r="A72" s="93" t="inlineStr">
+        <is>
+          <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="n"/>
+      <c r="C72" s="13" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="inlineStr">
-        <is>
-          <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
-        </is>
-      </c>
-      <c r="E73" s="101" t="n">
-        <v>14.1783354282636</v>
-      </c>
-      <c r="F73" s="101">
-        <f>F77/F75</f>
-        <v/>
-      </c>
-      <c r="G73" s="101">
-        <f>G77/G75</f>
-        <v/>
-      </c>
-      <c r="H73" s="101">
-        <f>H77/H75</f>
-        <v/>
-      </c>
-      <c r="I73" s="101">
-        <f>I77/I75</f>
-        <v/>
-      </c>
-      <c r="J73" s="101">
-        <f>J77/J75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74"/>
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>Selected exit EV/EBITDA (Gordon implied)</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="n"/>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>DCF: Gordon implied exit (TV / FY30 EBIT</t>
+        </is>
+      </c>
+      <c r="D74" s="19" t="n"/>
+      <c r="E74" s="94">
+        <f>E46</f>
+        <v/>
+      </c>
+      <c r="M74" s="95" t="n"/>
+    </row>
     <row r="75">
-      <c r="A75" s="93" t="inlineStr">
-        <is>
-          <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
-        </is>
-      </c>
-      <c r="B75" s="13" t="n"/>
-      <c r="C75" s="13" t="n"/>
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="E75" s="75">
+        <f>E41*E74</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="15" t="inlineStr">
-        <is>
-          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
-        </is>
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E76" s="75">
+        <f>E75/(1+Scenarios!$F$9)^J36</f>
+        <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="16" t="inlineStr">
-        <is>
-          <t>Selected exit EV/EBITDA (Gordon implied)</t>
-        </is>
-      </c>
-      <c r="B77" s="17" t="n"/>
-      <c r="C77" s="18" t="inlineStr">
-        <is>
-          <t>DCF: Gordon implied exit (TV / FY30 EBIT</t>
-        </is>
-      </c>
-      <c r="D77" s="19" t="n"/>
-      <c r="E77" s="94">
-        <f>E46</f>
-        <v/>
-      </c>
-      <c r="M77" s="95" t="n"/>
+      <c r="A77" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="E77" s="25">
+        <f>E39+E76</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="E78" s="75">
-        <f>E43*E77</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="16" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E79" s="75">
-        <f>E78/(1+Scenarios!$F$9)^J36</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A78" s="23" t="inlineStr">
+        <is>
+          <t>Implied value per share (exit method)</t>
+        </is>
+      </c>
+      <c r="E78" s="102">
+        <f>(E77+E46+E47)/E49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79"/>
     <row r="80">
-      <c r="A80" s="23" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="E80" s="25">
-        <f>E41+E79</f>
-        <v/>
-      </c>
+      <c r="A80" s="93" t="inlineStr">
+        <is>
+          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="n"/>
+      <c r="C80" s="13" t="n"/>
+      <c r="D80" s="13" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="23" t="inlineStr">
-        <is>
-          <t>Implied value per share (exit method)</t>
-        </is>
-      </c>
-      <c r="E81" s="102">
-        <f>(E80+E48+E49)/E51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" ht="28" customHeight="1"/>
+      <c r="A81" s="103" t="inlineStr"/>
+      <c r="B81" s="54" t="n"/>
+      <c r="C81" s="54" t="inlineStr">
+        <is>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="D81" s="54" t="n"/>
+    </row>
+    <row r="82" ht="28" customHeight="1">
+      <c r="A82" s="23" t="inlineStr">
+        <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B82" s="70" t="n"/>
+      <c r="C82" s="70">
+        <f>E83</f>
+        <v/>
+      </c>
+      <c r="D82" s="70" t="n"/>
+    </row>
     <row r="83">
-      <c r="A83" s="93" t="inlineStr">
-        <is>
-          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
-        </is>
-      </c>
-      <c r="B83" s="13" t="n"/>
-      <c r="C83" s="13" t="n"/>
-      <c r="D83" s="13" t="n"/>
+      <c r="A83" s="23" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA (implied vs selected)</t>
+        </is>
+      </c>
+      <c r="B83" s="104" t="n"/>
+      <c r="C83" s="104">
+        <f>E82</f>
+        <v/>
+      </c>
+      <c r="D83" s="104" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="103" t="inlineStr"/>
-      <c r="B84" s="54" t="n"/>
-      <c r="C84" s="54" t="inlineStr">
-        <is>
-          <t>Exit Multiple</t>
-        </is>
-      </c>
-      <c r="D84" s="54" t="n"/>
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value variance (%)</t>
+        </is>
+      </c>
+      <c r="B84" s="32" t="n"/>
+      <c r="C84" s="32" t="n"/>
+      <c r="D84" s="32" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
         <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B85" s="70" t="n"/>
-      <c r="C85" s="70">
-        <f>E83</f>
-        <v/>
-      </c>
-      <c r="D85" s="70" t="n"/>
+          <t>Implied share price</t>
+        </is>
+      </c>
+      <c r="B85" s="105" t="n"/>
+      <c r="C85" s="105">
+        <f>E86</f>
+        <v/>
+      </c>
+      <c r="D85" s="105" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="23" t="inlineStr">
-        <is>
-          <t>Exit EV/EBITDA (implied vs selected)</t>
-        </is>
-      </c>
-      <c r="B86" s="104" t="n"/>
-      <c r="C86" s="104">
-        <f>E82</f>
-        <v/>
-      </c>
-      <c r="D86" s="104" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value variance (%)</t>
-        </is>
-      </c>
-      <c r="B87" s="32" t="n"/>
-      <c r="C87" s="32" t="n"/>
-      <c r="D87" s="32" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="23" t="inlineStr">
-        <is>
-          <t>Implied share price</t>
-        </is>
-      </c>
-      <c r="B88" s="105" t="n"/>
-      <c r="C88" s="105">
-        <f>E86</f>
-        <v/>
-      </c>
-      <c r="D88" s="105" t="n"/>
-    </row>
+      <c r="A86" s="68" t="inlineStr">
+        <is>
+          <t>Sanity check: multiples within ±1.5 turns?</t>
+        </is>
+      </c>
+      <c r="B86" s="106" t="n"/>
+      <c r="C86" s="107">
+        <f>TEXT(D91,"0.0")&amp;"x spread vs Gordon-imp</f>
+        <v/>
+      </c>
+      <c r="D86" s="26" t="n"/>
+    </row>
+    <row r="87"/>
+    <row r="88"/>
     <row r="89">
-      <c r="A89" s="68" t="inlineStr">
-        <is>
-          <t>Sanity check: multiples within ±1.5 turns?</t>
-        </is>
-      </c>
-      <c r="B89" s="106" t="n"/>
-      <c r="C89" s="107">
-        <f>TEXT(D91,"0.0")&amp;"x spread vs Gordon-imp</f>
-        <v/>
-      </c>
-      <c r="D89" s="26" t="n"/>
-    </row>
-    <row r="90"/>
-    <row r="91"/>
+      <c r="A89" s="93" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="n"/>
+      <c r="C89" s="13" t="n"/>
+      <c r="D89" s="13" t="n"/>
+      <c r="E89" s="13" t="n"/>
+      <c r="F89" s="13" t="n"/>
+      <c r="G89" s="13" t="n"/>
+      <c r="H89" s="13" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="108" t="inlineStr">
+        <is>
+          <t>WACC \ g</t>
+        </is>
+      </c>
+      <c r="B90" s="17" t="n"/>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>FRED</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="n"/>
+      <c r="F90" s="109" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G90" s="109" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H90" s="109" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="I90" s="109" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="J90" s="109" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L90" s="95" t="inlineStr">
+        <is>
+          <t>Scenarios: terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="109" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="C91" s="95" t="inlineStr">
+        <is>
+          <t>Damodaran</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="n"/>
+      <c r="F91" s="110">
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="G91" s="110">
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="H91" s="110">
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="I91" s="110">
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="J91" s="110">
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="L91" s="95" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
     <row r="92">
-      <c r="A92" s="93" t="inlineStr">
-        <is>
-          <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
-        </is>
-      </c>
-      <c r="B92" s="13" t="n"/>
-      <c r="C92" s="13" t="n"/>
-      <c r="D92" s="13" t="n"/>
-      <c r="E92" s="13" t="n"/>
-      <c r="F92" s="13" t="n"/>
-      <c r="G92" s="13" t="n"/>
-      <c r="H92" s="13" t="n"/>
+      <c r="A92" s="109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D92" s="19" t="n"/>
+      <c r="F92" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="G92" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="H92" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="I92" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="J92" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="L92" s="95" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="108" t="inlineStr">
-        <is>
-          <t>WACC \ g</t>
-        </is>
-      </c>
-      <c r="B93" s="17" t="n"/>
-      <c r="C93" s="18" t="inlineStr">
-        <is>
-          <t>FRED</t>
-        </is>
+      <c r="A93" s="109" t="n">
+        <v>0.105</v>
       </c>
       <c r="D93" s="19" t="n"/>
-      <c r="F93" s="109" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="G93" s="109" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H93" s="109" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="I93" s="109" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="J93" s="109" t="n">
-        <v>0.03</v>
+      <c r="F93" s="110">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="G93" s="110">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="H93" s="111">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="I93" s="110">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E46+E47)/E49</f>
+        <v/>
+      </c>
+      <c r="J93" s="110">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E46+E47)/E49</f>
+        <v/>
       </c>
       <c r="L93" s="95" t="inlineStr">
         <is>
-          <t>Scenarios: terminal g</t>
+          <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="109" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="C94" s="95" t="inlineStr">
-        <is>
-          <t>Damodaran</t>
-        </is>
+        <v>0.11</v>
       </c>
       <c r="D94" s="19" t="n"/>
       <c r="F94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E48+E49)/E51</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="G94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E48+E49)/E51</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="H94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E48+E49)/E51</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="I94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E48+E49)/E51</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="J94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E48+E49)/E51</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="L94" s="95" t="inlineStr">
@@ -10616,27 +10669,27 @@
     </row>
     <row r="95">
       <c r="A95" s="109" t="n">
-        <v>0.1</v>
+        <v>0.115</v>
       </c>
       <c r="D95" s="19" t="n"/>
       <c r="F95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E48+E49)/E51</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="G95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E48+E49)/E51</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="H95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E48+E49)/E51</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="I95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E48+E49)/E51</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="J95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E48+E49)/E51</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E46+E47)/E49</f>
         <v/>
       </c>
       <c r="L95" s="95" t="inlineStr">
@@ -10646,113 +10699,22 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="109" t="n">
-        <v>0.105</v>
+      <c r="B96" s="17" t="n"/>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>WACC Tab</t>
+        </is>
       </c>
       <c r="D96" s="19" t="n"/>
-      <c r="F96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="G96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="H96" s="111">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="I96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="J96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
       <c r="L96" s="95" t="inlineStr">
         <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="109" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="D97" s="19" t="n"/>
-      <c r="F97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="G97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="H97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="I97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="J97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="L97" s="95" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="28" customHeight="1">
-      <c r="A98" s="109" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="D98" s="19" t="n"/>
-      <c r="F98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="G98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="H98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="I98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="J98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E48+E49)/E51</f>
-        <v/>
-      </c>
-      <c r="L98" s="95" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="28" customHeight="1">
-      <c r="B99" s="17" t="n"/>
-      <c r="C99" s="18" t="inlineStr">
-        <is>
-          <t>WACC Tab</t>
-        </is>
-      </c>
-      <c r="D99" s="19" t="n"/>
-      <c r="L99" s="95" t="inlineStr">
-        <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M99" s="19" t="n"/>
-    </row>
+      <c r="M96" s="19" t="n"/>
+    </row>
+    <row r="98" ht="28" customHeight="1"/>
+    <row r="99" ht="28" customHeight="1"/>
     <row r="100" ht="28" customHeight="1"/>
     <row r="101" ht="28" customHeight="1"/>
     <row r="102" ht="28" customHeight="1"/>
@@ -10760,68 +10722,67 @@
     <row r="104" ht="28" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
     <hyperlink ref="C4" location="'NOPAT Bridge'!A1"/>
     <hyperlink ref="D4" location="'Revenue Drivers'!A1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId33"/>
     <hyperlink ref="C30" location="'Scenarios'!A105"/>
     <hyperlink ref="C31" location="'Scenarios'!A110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId35"/>
     <hyperlink ref="C33" location="'Scenarios'!A120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId44"/>
     <hyperlink ref="C82" location="'DCF'!E46"/>
     <hyperlink ref="M82" location="'Comps'!A45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId45"/>
     <hyperlink ref="L98" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId46"/>
     <hyperlink ref="L99" location="'WACC'!E41"/>
     <hyperlink ref="L100" location="'WACC'!E41"/>
     <hyperlink ref="L101" location="'WACC'!E41"/>
     <hyperlink ref="L102" location="'WACC'!E41"/>
     <hyperlink ref="L103" location="'WACC'!E41"/>
     <hyperlink ref="C104" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>